<commit_message>
Facility Yield Analysis v2: header styling on the lender/Zed view row; fix pts number format (showed 0.1 instead of 5.3)
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261027.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261027.xlsx
@@ -48,13 +48,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000%"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="168" formatCode="0.0&quot; pts&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -119,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,7 +144,6 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -1660,31 +1658,32 @@
           <t xml:space="preserve">  FPD cost = difference, borne by Zed if FPD receivables are ineligible</t>
         </is>
       </c>
-      <c r="C26" s="20">
+      <c r="C26" s="13">
         <f>C25-C23</f>
         <v/>
       </c>
     </row>
     <row r="27"/>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Net yield and excess spread</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="14" t="inlineStr">
+    <row r="28"/>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Net yield and excess spread — points of average receivables per year</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Lender's view (pool ex-FPD)</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Zed's view (all losses)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Comment</t>
         </is>
       </c>
     </row>
@@ -1839,11 +1838,11 @@
           <t>Coverage = net yield ÷ cost of funds</t>
         </is>
       </c>
-      <c r="B38" s="21">
+      <c r="B38" s="20">
         <f>B32/(B33+B34+B35)</f>
         <v/>
       </c>
-      <c r="C38" s="21">
+      <c r="C38" s="20">
         <f>C32/(C33+C34+C35)</f>
         <v/>
       </c>
@@ -1879,11 +1878,11 @@
           <t>Headroom: breakeven ÷ current loss rate</t>
         </is>
       </c>
-      <c r="B40" s="21">
+      <c r="B40" s="20">
         <f>B39/C22</f>
         <v/>
       </c>
-      <c r="C40" s="21">
+      <c r="C40" s="20">
         <f>C39/C24</f>
         <v/>
       </c>
@@ -1915,7 +1914,7 @@
     </row>
     <row r="42"/>
     <row r="43" ht="48" customHeight="1">
-      <c r="A43" s="22" t="inlineStr">
+      <c r="A43" s="21" t="inlineStr">
         <is>
           <t>Read: the lender underwrites the left column (its pool excludes FPD receivables, which Zed repurchases); Zed lives in the right column. Today the FPD cost (row 26) consumes nearly all of Zed's excess spread — the new fraud controls are the margin. Frictions (withholding, hedge) are placeholders at 0 and would come off Zed's column.</t>
         </is>
@@ -1957,7 +1956,7 @@
       </c>
     </row>
     <row r="2" ht="64" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Model: transacting and installment balances held at Q3 levels; revolving balance scaled to hit the target share of balances; revolving interest = Q3 monthly rate × 12 on the revolving balance; purchase volume, pay-a-friend, interchange, installment charges and late fees held in pesos (spend- and conversion-driven, not balance-driven); principal flow therefore held, so turnover falls as the book grows and the same loss rate on originations becomes a smaller loss on balances. Cost of funds = coupon × advance rate; withholding and hedge at their Inputs values (0 unless set).</t>
         </is>
@@ -1989,7 +1988,7 @@
         <f>rev_int/(bal_rev*months)</f>
         <v/>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>rev_int ÷ Σ monthly revolving balances (Jul–Sep) — 2.44%; BSP cap 3%</t>
         </is>
@@ -2016,7 +2015,7 @@
         <f>(bal_tra+bal_inst)/bal_tot*avg_rec</f>
         <v/>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>held constant across scenarios</t>
         </is>
@@ -2032,7 +2031,7 @@
         <f>flow*12/months</f>
         <v/>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>held constant</t>
         </is>
@@ -2048,7 +2047,7 @@
         <f>(interchange+inst_int+upfront+late)*12/months</f>
         <v/>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>held constant in pesos</t>
         </is>
@@ -2064,7 +2063,7 @@
         <f>coupon*advance*wht/(1-wht)+hedge*advance</f>
         <v/>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>0 unless set on Inputs</t>
         </is>
@@ -2077,7 +2076,7 @@
           <t>Revolving share of balances = Q3 average</t>
         </is>
       </c>
-      <c r="B12" s="25">
+      <c r="B12" s="24">
         <f>bal_rev/bal_tot</f>
         <v/>
       </c>
@@ -2151,22 +2150,22 @@
           <t>Excess spread, pts of receivables — coupon ↓ / loss rate →</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="25" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="25" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
       </c>
-      <c r="D19" s="26" t="inlineStr">
+      <c r="D19" s="25" t="inlineStr">
         <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E19" s="26" t="inlineStr">
+      <c r="E19" s="25" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
@@ -2176,12 +2175,12 @@
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H19" s="26" t="inlineStr">
+      <c r="H19" s="25" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I19" s="26" t="inlineStr">
+      <c r="I19" s="25" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
@@ -2193,19 +2192,19 @@
           <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B20" s="20">
+      <c r="B20" s="13">
         <f>$B$15-L_x90*$B$17-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C20" s="20">
+      <c r="C20" s="13">
         <f>$B$15-L_all90*$B$17-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="13">
         <f>$B$15-L_life90x*$B$17-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E20" s="20">
+      <c r="E20" s="13">
         <f>$B$15-L_life90*$B$17-0.15*advance-$B$10</f>
         <v/>
       </c>
@@ -2224,19 +2223,19 @@
           <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B21" s="20">
+      <c r="B21" s="13">
         <f>$B$15-L_x90*$B$17-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="13">
         <f>$B$15-L_all90*$B$17-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="13">
         <f>$B$15-L_life90x*$B$17-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="13">
         <f>$B$15-L_life90*$B$17-0.17*advance-$B$10</f>
         <v/>
       </c>
@@ -2255,19 +2254,19 @@
           <t>Coupon 19% (cost on receivables = 19% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B22" s="20">
+      <c r="B22" s="13">
         <f>$B$15-L_x90*$B$17-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C22" s="20">
+      <c r="C22" s="13">
         <f>$B$15-L_all90*$B$17-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="13">
         <f>$B$15-L_life90x*$B$17-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="13">
         <f>$B$15-L_life90*$B$17-0.19*advance-$B$10</f>
         <v/>
       </c>
@@ -2306,19 +2305,19 @@
           <t xml:space="preserve">  Excess spread, pts of receivables</t>
         </is>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="13">
         <f>$B$15-L_x90*$B$17-0.19*B24-$B$10</f>
         <v/>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="13">
         <f>$B$15-L_x90*$B$17-0.19*C24-$B$10</f>
         <v/>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="13">
         <f>$B$15-L_x90*$B$17-0.19*D24-$B$10</f>
         <v/>
       </c>
-      <c r="E25" s="20">
+      <c r="E25" s="13">
         <f>$B$15-L_x90*$B$17-0.19*E24-$B$10</f>
         <v/>
       </c>
@@ -2329,19 +2328,19 @@
           <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
         </is>
       </c>
-      <c r="B26" s="21">
+      <c r="B26" s="20">
         <f>($B$15-L_x90*$B$17)/(0.19*B24+$B$10)</f>
         <v/>
       </c>
-      <c r="C26" s="21">
+      <c r="C26" s="20">
         <f>($B$15-L_x90*$B$17)/(0.19*C24+$B$10)</f>
         <v/>
       </c>
-      <c r="D26" s="21">
+      <c r="D26" s="20">
         <f>($B$15-L_x90*$B$17)/(0.19*D24+$B$10)</f>
         <v/>
       </c>
-      <c r="E26" s="21">
+      <c r="E26" s="20">
         <f>($B$15-L_x90*$B$17)/(0.19*E24+$B$10)</f>
         <v/>
       </c>
@@ -2376,7 +2375,7 @@
           <t>Revolving share of balances = 50%</t>
         </is>
       </c>
-      <c r="B29" s="25" t="n">
+      <c r="B29" s="24" t="n">
         <v>0.5</v>
       </c>
       <c r="C29" s="5" t="n"/>
@@ -2449,22 +2448,22 @@
           <t>Excess spread, pts of receivables — coupon ↓ / loss rate →</t>
         </is>
       </c>
-      <c r="B36" s="26" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C36" s="26" t="inlineStr">
+      <c r="C36" s="25" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
       </c>
-      <c r="D36" s="26" t="inlineStr">
+      <c r="D36" s="25" t="inlineStr">
         <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E36" s="26" t="inlineStr">
+      <c r="E36" s="25" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
@@ -2474,12 +2473,12 @@
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H36" s="26" t="inlineStr">
+      <c r="H36" s="25" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I36" s="26" t="inlineStr">
+      <c r="I36" s="25" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
@@ -2491,19 +2490,19 @@
           <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B37" s="20">
+      <c r="B37" s="13">
         <f>$B$32-L_x90*$B$34-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C37" s="20">
+      <c r="C37" s="13">
         <f>$B$32-L_all90*$B$34-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D37" s="20">
+      <c r="D37" s="13">
         <f>$B$32-L_life90x*$B$34-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E37" s="20">
+      <c r="E37" s="13">
         <f>$B$32-L_life90*$B$34-0.15*advance-$B$10</f>
         <v/>
       </c>
@@ -2522,19 +2521,19 @@
           <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B38" s="20">
+      <c r="B38" s="13">
         <f>$B$32-L_x90*$B$34-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C38" s="20">
+      <c r="C38" s="13">
         <f>$B$32-L_all90*$B$34-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D38" s="20">
+      <c r="D38" s="13">
         <f>$B$32-L_life90x*$B$34-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E38" s="20">
+      <c r="E38" s="13">
         <f>$B$32-L_life90*$B$34-0.17*advance-$B$10</f>
         <v/>
       </c>
@@ -2553,19 +2552,19 @@
           <t>Coupon 19% (cost on receivables = 19% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B39" s="20">
+      <c r="B39" s="13">
         <f>$B$32-L_x90*$B$34-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C39" s="20">
+      <c r="C39" s="13">
         <f>$B$32-L_all90*$B$34-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D39" s="20">
+      <c r="D39" s="13">
         <f>$B$32-L_life90x*$B$34-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E39" s="20">
+      <c r="E39" s="13">
         <f>$B$32-L_life90*$B$34-0.19*advance-$B$10</f>
         <v/>
       </c>
@@ -2604,19 +2603,19 @@
           <t xml:space="preserve">  Excess spread, pts of receivables</t>
         </is>
       </c>
-      <c r="B42" s="20">
+      <c r="B42" s="13">
         <f>$B$32-L_x90*$B$34-0.19*B41-$B$10</f>
         <v/>
       </c>
-      <c r="C42" s="20">
+      <c r="C42" s="13">
         <f>$B$32-L_x90*$B$34-0.19*C41-$B$10</f>
         <v/>
       </c>
-      <c r="D42" s="20">
+      <c r="D42" s="13">
         <f>$B$32-L_x90*$B$34-0.19*D41-$B$10</f>
         <v/>
       </c>
-      <c r="E42" s="20">
+      <c r="E42" s="13">
         <f>$B$32-L_x90*$B$34-0.19*E41-$B$10</f>
         <v/>
       </c>
@@ -2627,19 +2626,19 @@
           <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
         </is>
       </c>
-      <c r="B43" s="21">
+      <c r="B43" s="20">
         <f>($B$32-L_x90*$B$34)/(0.19*B41+$B$10)</f>
         <v/>
       </c>
-      <c r="C43" s="21">
+      <c r="C43" s="20">
         <f>($B$32-L_x90*$B$34)/(0.19*C41+$B$10)</f>
         <v/>
       </c>
-      <c r="D43" s="21">
+      <c r="D43" s="20">
         <f>($B$32-L_x90*$B$34)/(0.19*D41+$B$10)</f>
         <v/>
       </c>
-      <c r="E43" s="21">
+      <c r="E43" s="20">
         <f>($B$32-L_x90*$B$34)/(0.19*E41+$B$10)</f>
         <v/>
       </c>
@@ -2674,7 +2673,7 @@
           <t>Revolving share of balances = 55%</t>
         </is>
       </c>
-      <c r="B46" s="25" t="n">
+      <c r="B46" s="24" t="n">
         <v>0.55</v>
       </c>
       <c r="C46" s="5" t="n"/>
@@ -2747,22 +2746,22 @@
           <t>Excess spread, pts of receivables — coupon ↓ / loss rate →</t>
         </is>
       </c>
-      <c r="B53" s="26" t="inlineStr">
+      <c r="B53" s="25" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C53" s="26" t="inlineStr">
+      <c r="C53" s="25" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
       </c>
-      <c r="D53" s="26" t="inlineStr">
+      <c r="D53" s="25" t="inlineStr">
         <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E53" s="26" t="inlineStr">
+      <c r="E53" s="25" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
@@ -2772,12 +2771,12 @@
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H53" s="26" t="inlineStr">
+      <c r="H53" s="25" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I53" s="26" t="inlineStr">
+      <c r="I53" s="25" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
@@ -2789,19 +2788,19 @@
           <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B54" s="20">
+      <c r="B54" s="13">
         <f>$B$49-L_x90*$B$51-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C54" s="20">
+      <c r="C54" s="13">
         <f>$B$49-L_all90*$B$51-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D54" s="20">
+      <c r="D54" s="13">
         <f>$B$49-L_life90x*$B$51-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E54" s="20">
+      <c r="E54" s="13">
         <f>$B$49-L_life90*$B$51-0.15*advance-$B$10</f>
         <v/>
       </c>
@@ -2820,19 +2819,19 @@
           <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B55" s="20">
+      <c r="B55" s="13">
         <f>$B$49-L_x90*$B$51-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C55" s="20">
+      <c r="C55" s="13">
         <f>$B$49-L_all90*$B$51-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D55" s="20">
+      <c r="D55" s="13">
         <f>$B$49-L_life90x*$B$51-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E55" s="20">
+      <c r="E55" s="13">
         <f>$B$49-L_life90*$B$51-0.17*advance-$B$10</f>
         <v/>
       </c>
@@ -2851,19 +2850,19 @@
           <t>Coupon 19% (cost on receivables = 19% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B56" s="20">
+      <c r="B56" s="13">
         <f>$B$49-L_x90*$B$51-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C56" s="20">
+      <c r="C56" s="13">
         <f>$B$49-L_all90*$B$51-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D56" s="20">
+      <c r="D56" s="13">
         <f>$B$49-L_life90x*$B$51-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E56" s="20">
+      <c r="E56" s="13">
         <f>$B$49-L_life90*$B$51-0.19*advance-$B$10</f>
         <v/>
       </c>
@@ -2902,19 +2901,19 @@
           <t xml:space="preserve">  Excess spread, pts of receivables</t>
         </is>
       </c>
-      <c r="B59" s="20">
+      <c r="B59" s="13">
         <f>$B$49-L_x90*$B$51-0.19*B58-$B$10</f>
         <v/>
       </c>
-      <c r="C59" s="20">
+      <c r="C59" s="13">
         <f>$B$49-L_x90*$B$51-0.19*C58-$B$10</f>
         <v/>
       </c>
-      <c r="D59" s="20">
+      <c r="D59" s="13">
         <f>$B$49-L_x90*$B$51-0.19*D58-$B$10</f>
         <v/>
       </c>
-      <c r="E59" s="20">
+      <c r="E59" s="13">
         <f>$B$49-L_x90*$B$51-0.19*E58-$B$10</f>
         <v/>
       </c>
@@ -2925,19 +2924,19 @@
           <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
         </is>
       </c>
-      <c r="B60" s="21">
+      <c r="B60" s="20">
         <f>($B$49-L_x90*$B$51)/(0.19*B58+$B$10)</f>
         <v/>
       </c>
-      <c r="C60" s="21">
+      <c r="C60" s="20">
         <f>($B$49-L_x90*$B$51)/(0.19*C58+$B$10)</f>
         <v/>
       </c>
-      <c r="D60" s="21">
+      <c r="D60" s="20">
         <f>($B$49-L_x90*$B$51)/(0.19*D58+$B$10)</f>
         <v/>
       </c>
-      <c r="E60" s="21">
+      <c r="E60" s="20">
         <f>($B$49-L_x90*$B$51)/(0.19*E58+$B$10)</f>
         <v/>
       </c>
@@ -2972,7 +2971,7 @@
           <t>Revolving share of balances = 60%</t>
         </is>
       </c>
-      <c r="B63" s="25" t="n">
+      <c r="B63" s="24" t="n">
         <v>0.6</v>
       </c>
       <c r="C63" s="5" t="n"/>
@@ -3045,22 +3044,22 @@
           <t>Excess spread, pts of receivables — coupon ↓ / loss rate →</t>
         </is>
       </c>
-      <c r="B70" s="26" t="inlineStr">
+      <c r="B70" s="25" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C70" s="26" t="inlineStr">
+      <c r="C70" s="25" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
       </c>
-      <c r="D70" s="26" t="inlineStr">
+      <c r="D70" s="25" t="inlineStr">
         <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E70" s="26" t="inlineStr">
+      <c r="E70" s="25" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
@@ -3070,12 +3069,12 @@
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H70" s="26" t="inlineStr">
+      <c r="H70" s="25" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I70" s="26" t="inlineStr">
+      <c r="I70" s="25" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
@@ -3087,19 +3086,19 @@
           <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B71" s="20">
+      <c r="B71" s="13">
         <f>$B$66-L_x90*$B$68-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C71" s="20">
+      <c r="C71" s="13">
         <f>$B$66-L_all90*$B$68-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D71" s="20">
+      <c r="D71" s="13">
         <f>$B$66-L_life90x*$B$68-0.15*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E71" s="20">
+      <c r="E71" s="13">
         <f>$B$66-L_life90*$B$68-0.15*advance-$B$10</f>
         <v/>
       </c>
@@ -3118,19 +3117,19 @@
           <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B72" s="20">
+      <c r="B72" s="13">
         <f>$B$66-L_x90*$B$68-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C72" s="20">
+      <c r="C72" s="13">
         <f>$B$66-L_all90*$B$68-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D72" s="20">
+      <c r="D72" s="13">
         <f>$B$66-L_life90x*$B$68-0.17*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E72" s="20">
+      <c r="E72" s="13">
         <f>$B$66-L_life90*$B$68-0.17*advance-$B$10</f>
         <v/>
       </c>
@@ -3149,19 +3148,19 @@
           <t>Coupon 19% (cost on receivables = 19% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B73" s="20">
+      <c r="B73" s="13">
         <f>$B$66-L_x90*$B$68-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="C73" s="20">
+      <c r="C73" s="13">
         <f>$B$66-L_all90*$B$68-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="D73" s="20">
+      <c r="D73" s="13">
         <f>$B$66-L_life90x*$B$68-0.19*advance-$B$10</f>
         <v/>
       </c>
-      <c r="E73" s="20">
+      <c r="E73" s="13">
         <f>$B$66-L_life90*$B$68-0.19*advance-$B$10</f>
         <v/>
       </c>
@@ -3200,19 +3199,19 @@
           <t xml:space="preserve">  Excess spread, pts of receivables</t>
         </is>
       </c>
-      <c r="B76" s="20">
+      <c r="B76" s="13">
         <f>$B$66-L_x90*$B$68-0.19*B75-$B$10</f>
         <v/>
       </c>
-      <c r="C76" s="20">
+      <c r="C76" s="13">
         <f>$B$66-L_x90*$B$68-0.19*C75-$B$10</f>
         <v/>
       </c>
-      <c r="D76" s="20">
+      <c r="D76" s="13">
         <f>$B$66-L_x90*$B$68-0.19*D75-$B$10</f>
         <v/>
       </c>
-      <c r="E76" s="20">
+      <c r="E76" s="13">
         <f>$B$66-L_x90*$B$68-0.19*E75-$B$10</f>
         <v/>
       </c>
@@ -3223,19 +3222,19 @@
           <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
         </is>
       </c>
-      <c r="B77" s="21">
+      <c r="B77" s="20">
         <f>($B$66-L_x90*$B$68)/(0.19*B75+$B$10)</f>
         <v/>
       </c>
-      <c r="C77" s="21">
+      <c r="C77" s="20">
         <f>($B$66-L_x90*$B$68)/(0.19*C75+$B$10)</f>
         <v/>
       </c>
-      <c r="D77" s="21">
+      <c r="D77" s="20">
         <f>($B$66-L_x90*$B$68)/(0.19*D75+$B$10)</f>
         <v/>
       </c>
-      <c r="E77" s="21">
+      <c r="E77" s="20">
         <f>($B$66-L_x90*$B$68)/(0.19*E75+$B$10)</f>
         <v/>
       </c>
@@ -3265,7 +3264,7 @@
     </row>
     <row r="79"/>
     <row r="80" ht="64" customHeight="1">
-      <c r="A80" s="22" t="inlineStr">
+      <c r="A80" s="21" t="inlineStr">
         <is>
           <t>Calibration: the Q3-share block rebuilds revolving interest as rate × scaled revolving balance, so its gross yield (32.1%) sits 0.25 pts under the Q3 sheet (32.4%) and its base-case excess spread reads 5.4 vs 5.6 pts; the gap is the same in every block and does not affect the comparisons. Read across: base case = Q3 share (41.8%), ex-FPD ≥90 loss, 19% coupon, 80% advance → the first cell of the first grid. The second loss column is the tape-level number Accial will compute before any FPD carve-out — at 19% it is close to zero excess spread, which is why FPD ineligibility has to be structural. Moving to 50–60% revolving raises interest yield faster than it dilutes interchange and lowers turnover (so loss on receivables falls): read down the first column of each block. Each 2 pts of coupon ≈ 1.6 pts of excess spread at 80% advance; each 5 pts of advance rate ≈ 1 pt.</t>
         </is>

</xml_diff>

<commit_message>
Facility Yield Analysis v2: revolving interest as 3.05% on interest-bearing balance × 0.80 bucket ratio (growth/timing), ratio sensitivity added
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261027.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261027.xlsx
@@ -26,21 +26,32 @@
     <definedName name="bal_tra">Inputs!$B$17</definedName>
     <definedName name="bal_inst">Inputs!$B$18</definedName>
     <definedName name="bal_tot">Inputs!$B$19</definedName>
-    <definedName name="purch">Inputs!$B$21</definedName>
-    <definedName name="paf">Inputs!$B$22</definedName>
-    <definedName name="flow">Inputs!$B$23</definedName>
-    <definedName name="orig_stmt">Inputs!$B$24</definedName>
-    <definedName name="L_x90">Inputs!$B$26</definedName>
-    <definedName name="L_all90">Inputs!$B$27</definedName>
-    <definedName name="L_fpd90">Inputs!$B$28</definedName>
-    <definedName name="L_life90x">Inputs!$B$29</definedName>
-    <definedName name="L_life90">Inputs!$B$30</definedName>
-    <definedName name="L_x16">Inputs!$B$31</definedName>
-    <definedName name="coupon">Inputs!$B$33</definedName>
-    <definedName name="advance">Inputs!$B$34</definedName>
-    <definedName name="wht">Inputs!$B$35</definedName>
-    <definedName name="hedge">Inputs!$B$36</definedName>
-    <definedName name="fx">Inputs!$B$37</definedName>
+    <definedName name="pib">Inputs!$B$20</definedName>
+    <definedName name="rate_ib">Inputs!$B$21</definedName>
+    <definedName name="ratio_obs">Inputs!$B$22</definedName>
+    <definedName name="ratio_scn">Inputs!$B$23</definedName>
+    <definedName name="purch">Inputs!$B$25</definedName>
+    <definedName name="paf">Inputs!$B$26</definedName>
+    <definedName name="flow">Inputs!$B$27</definedName>
+    <definedName name="orig_stmt">Inputs!$B$28</definedName>
+    <definedName name="L_x90">Inputs!$B$30</definedName>
+    <definedName name="L_all90">Inputs!$B$31</definedName>
+    <definedName name="L_fpd90">Inputs!$B$32</definedName>
+    <definedName name="L_life90x">Inputs!$B$33</definedName>
+    <definedName name="L_life90">Inputs!$B$34</definedName>
+    <definedName name="L_x16">Inputs!$B$35</definedName>
+    <definedName name="coupon">Inputs!$B$37</definedName>
+    <definedName name="advance">Inputs!$B$38</definedName>
+    <definedName name="wht">Inputs!$B$39</definedName>
+    <definedName name="hedge">Inputs!$B$40</definedName>
+    <definedName name="fx">Inputs!$B$41</definedName>
+    <definedName name="s_rate">Scenarios!$B$5</definedName>
+    <definedName name="s_ratio">Scenarios!$B$6</definedName>
+    <definedName name="s_share">Scenarios!$B$7</definedName>
+    <definedName name="s_nonrev">Scenarios!$B$8</definedName>
+    <definedName name="s_flow">Scenarios!$B$9</definedName>
+    <definedName name="s_other">Scenarios!$B$10</definedName>
+    <definedName name="s_fric">Scenarios!$B$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48,12 +59,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="0.000%"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="168" formatCode="0.00&quot;x&quot;"/>
+  <numFmts count="6">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.000%"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -118,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,18 +144,19 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -151,10 +164,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -920,237 +935,239 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>FLOWS — Jul–Sep 2026 (calendar month)</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Interest-bearing balance on revolver statements, Σ Jul–Sep (purchase_interest_balance)</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>186570217.4</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PHP</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>BigQuery public_statements.purchase_interest_balance, on-cycle statements closing Jul–Sep 2026 with interest_charged &gt; 0 (query 2026-10-27)</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>The balance the 3%/month APR was actually applied to (average revolved balance over the cycle). Σ of the three months' revolving-bucket ending balances is 232,897,157 on the same statements.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Purchase volume settled (Mastercard, net of returns)</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="n">
-        <v>448499545.15</v>
+          <t>Monthly rate on the interest-bearing balance</t>
+        </is>
+      </c>
+      <c r="B21" s="9">
+        <f>rev_int/pib</f>
+        <v/>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>ratio</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>KPI Dashboard Monthly r127, Jul–Sep</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>127,249,656.88 + 130,388,896.48 + 190,860,991.79 — interchange base</t>
+          <t>3.05%/month ≈ 36.5% APR — the pricing. Statement-side interest (5,720,564) gives 3.07%; the 0.7% gap to dashboard r55 is cycle vs calendar</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Pay-a-friend transfers</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="n">
-        <v>8350000</v>
+          <t>Interest-bearing balance ÷ revolving-bucket ending balance, observed Q3</t>
+        </is>
+      </c>
+      <c r="B22" s="10">
+        <f>pib/(bal_rev*months)</f>
+        <v/>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>ratio</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>source-reports/pay_a_friend_transfers_by_month_2026-01_to_2026-09_10272026.csv (i2c C2C Transfer-Others, positive legs, response 00)</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>2.73M + 2.97M + 2.65M — no interchange; is principal</t>
+          <t>0.80. Interest is charged on the average revolved balance over the cycle; the bucket is the end-of-cycle balance, which includes the cycle's new purchases (₱101.5M of the ₱232.9M, accruing only from their posting date) and the billed interest/fee lines (₱7.7M). In a book growing ~15%/month the end-of-cycle balance runs ~25% above the cycle average. Timing/growth, not pricing</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Principal flow (purchase volume + pay-a-friend)</t>
-        </is>
-      </c>
-      <c r="B23" s="8">
-        <f>purch+paf</f>
+          <t>Interest-bearing ÷ bucket ratio used in Scenarios</t>
+        </is>
+      </c>
+      <c r="B23" s="10">
+        <f>ratio_obs</f>
         <v/>
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>assumption (defaults to observed)</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Override to test steady state: as growth slows the ratio rises toward ~0.9–0.95 (only the fee/interest lines and intra-cycle purchase timing remain outside the interest-bearing balance). Sensitivity table at the bottom of Scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>FLOWS — Jul–Sep 2026 (calendar month)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Purchase volume settled (Mastercard, net of returns)</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n">
+        <v>448499545.15</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>PHP</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Loss base, calendar-dated to match the denominator</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Principal originated, statement-month basis (reference)</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="n">
-        <v>442733819.38</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>PHP</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>source-reports/vintage_loss_by_origination_month_10262026.csv, originated_principal_php, 2026-07/08/09</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Base on which the loss rates below were measured; differs from the calendar flow by ~2 weeks of timing (agree within 1.2% over Jan–Sep)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>LOSS RATES — delinquent principal ÷ originated principal, denominator seasoned to the DPD cut</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>KPI Dashboard Monthly r127, Jul–Sep</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>127,249,656.88 + 130,388,896.48 + 190,860,991.79 — interchange base</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Since Jan 2026, ≥90 DPD, ex-FPD — BASE CASE</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="n">
-        <v>0.01152</v>
+          <t>Pay-a-friend transfers</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>8350000</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>PHP</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>source-reports/vintage_loss_seasoned_16_30_60_90_by_origination_month_10272026.csv, Σ d90x ÷ Σ s90x over 2026-01…09</t>
+          <t>source-reports/pay_a_friend_transfers_by_month_2026-01_to_2026-09_10272026.csv (i2c C2C Transfer-Others, positive legs, response 00)</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>₱6,668,630 ÷ ₱578,837,337. Steve 2026-10-27: ≥90 DPD is the loss proxy; FPD (first statement missed, never paid) excluded as fraud, managed separately by new controls</t>
+          <t>2.73M + 2.97M + 2.65M — no interchange; is principal</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Since Jan 2026, ≥90 DPD, all accounts</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="n">
-        <v>0.016812</v>
+          <t>Principal flow (purchase volume + pay-a-friend)</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>purch+paf</f>
+        <v/>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>PHP</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>same file, Σ d90 ÷ Σ s90</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>₱9,787,190 ÷ ₱582,182,780 — what Accial will compute from the tape before any FPD carve-out</t>
+          <t>Loss base, calendar-dated to match the denominator</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  of which first-payment default</t>
-        </is>
-      </c>
-      <c r="B28" s="9">
-        <f>L_all90-L_x90</f>
-        <v/>
+          <t>Principal originated, statement-month basis (reference)</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>442733819.38</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>PHP</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>source-reports/vintage_loss_by_origination_month_10262026.csv, originated_principal_php, 2026-07/08/09</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Borne by Zed outside the facility if FPD receivables are ineligible / repurchased</t>
+          <t>Base on which the loss rates below were measured; differs from the calendar flow by ~2 weeks of timing (agree within 1.2% over Jan–Sep)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Lifetime (Jan 2024–Sep 2026), ≥90 DPD, ex-FPD</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="n">
-        <v>0.013418</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>ratio</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>same file, lifetime rows</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Includes V1-model 2025 vintages</t>
-        </is>
-      </c>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>LOSS RATES — delinquent principal ÷ originated principal, denominator seasoned to the DPD cut</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Lifetime, ≥90 DPD, all accounts</t>
+          <t>Since Jan 2026, ≥90 DPD, ex-FPD — BASE CASE</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
-        <v>0.01922</v>
+        <v>0.01152</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1159,23 +1176,23 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>same file</t>
+          <t>source-reports/vintage_loss_seasoned_16_30_60_90_by_origination_month_10272026.csv, Σ d90x ÷ Σ s90x over 2026-01…09</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Most conservative citable figure</t>
+          <t>₱6,668,630 ÷ ₱578,837,337. Steve 2026-10-27: ≥90 DPD is the loss proxy; FPD (first statement missed, never paid) excluded as fraud, managed separately by new controls</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Since Jan 2026, &gt;15 DPD, ex-FPD (reference)</t>
+          <t>Since Jan 2026, ≥90 DPD, all accounts</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>0.01111</v>
+        <v>0.016812</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1184,34 +1201,49 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>same file</t>
+          <t>same file, Σ d90 ÷ Σ s90</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>16-day seasoned; close to L_x90 because almost nothing cures once &gt;15 DPD</t>
+          <t>₱9,787,190 ÷ ₱582,182,780 — what Accial will compute from the tape before any FPD carve-out</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>FACILITY ASSUMPTIONS</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n"/>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="5" t="n"/>
-      <c r="E32" s="5" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which first-payment default</t>
+        </is>
+      </c>
+      <c r="B32" s="9">
+        <f>L_all90-L_x90</f>
+        <v/>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Borne by Zed outside the facility if FPD receivables are ineligible / repurchased</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Coupon (all-in interest on drawn amount)</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="n">
-        <v>0.19</v>
+          <t>Lifetime (Jan 2024–Sep 2026), ≥90 DPD, ex-FPD</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>0.013418</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1220,23 +1252,23 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Assumption — Steve ('high teens')</t>
+          <t>same file, lifetime rows</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Scenario grid runs 15/17/19%</t>
+          <t>Includes V1-model 2025 vintages</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Advance rate (drawn ÷ eligible receivables)</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="n">
-        <v>0.8</v>
+          <t>Lifetime, ≥90 DPD, all accounts</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>0.01922</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1245,23 +1277,23 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Assumption — market 70–85% (structure note §3.3)</t>
+          <t>same file</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Cost of funds on receivables = coupon × advance; scenario runs 70/75/80%</t>
+          <t>Most conservative citable figure</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Withholding tax on coupon, if grossed up (placeholder)</t>
+          <t>Since Jan 2026, &gt;15 DPD, ex-FPD (reference)</t>
         </is>
       </c>
       <c r="B35" s="9" t="n">
-        <v>0</v>
+        <v>0.01111</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1270,60 +1302,146 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>NOT SIZED — PH 20% FWT / 15% US treaty (verification-notes/PH tax)</t>
+          <t>same file</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Set to 0 until the structure fixes who bears it; cost if grossed up = coupon × advance × wht ÷ (1 − wht)</t>
+          <t>16-day seasoned; close to L_x90 because almost nothing cures once &gt;15 DPD</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>FX hedge cost, % of drawn per year (placeholder)</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>ratio</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>NOT SIZED</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>USD facility vs PHP receivables; PHP/USD forward points — size before pricing</t>
-        </is>
-      </c>
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>FACILITY ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Coupon (all-in interest on drawn amount)</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Assumption — Steve ('high teens')</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Scenario grid runs 15/17/19%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Advance rate (drawn ÷ eligible receivables)</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Assumption — market 70–85% (structure note §3.3)</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Cost of funds on receivables = coupon × advance; scenario runs 70/75/80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Withholding tax on coupon, if grossed up (placeholder)</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>NOT SIZED — PH 20% FWT / 15% US treaty (verification-notes/PH tax)</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Set to 0 until the structure fixes who bears it; cost if grossed up = coupon × advance × wht ÷ (1 − wht)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>FX hedge cost, % of drawn per year (placeholder)</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>NOT SIZED</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>USD facility vs PHP receivables; PHP/USD forward points — size before pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>FX PHP per USD</t>
         </is>
       </c>
-      <c r="B37" s="11" t="n">
+      <c r="B41" s="12" t="n">
         <v>55.8</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>ratio</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>KPI Dashboard Monthly C2</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>Display only</t>
         </is>
@@ -1395,17 +1513,17 @@
           <t>Revolving interest</t>
         </is>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="13">
         <f>rev_int</f>
         <v/>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="14">
         <f>B5*12/months/avg_rec</f>
         <v/>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>2.44%/month on the revolving balance (rev_int ÷ Σ monthly revolving balances) — see Scenarios!B5</t>
+          <t>Charged at 3.05%/month (36.5% APR) on the interest-bearing balance (Inputs: rate_ib). Divided by the revolving bucket's end-of-cycle balance it reads 2.44%, because that balance includes the cycle's new purchases and billed lines not yet in the interest base — a growth/timing effect, not a lower rate</t>
         </is>
       </c>
     </row>
@@ -1415,11 +1533,11 @@
           <t>Installment interest + upfront fees</t>
         </is>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="13">
         <f>inst_int+upfront</f>
         <v/>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="14">
         <f>B6*12/months/avg_rec</f>
         <v/>
       </c>
@@ -1430,26 +1548,26 @@
           <t>Late payment fees</t>
         </is>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="13">
         <f>late</f>
         <v/>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="14">
         <f>B7*12/months/avg_rec</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Interest and fees</t>
         </is>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <f>SUM(B5:B7)</f>
         <v/>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="17">
         <f>B8*12/months/avg_rec</f>
         <v/>
       </c>
@@ -1476,7 +1594,7 @@
           <t>Purchase volume settled</t>
         </is>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="13">
         <f>purch</f>
         <v/>
       </c>
@@ -1487,7 +1605,7 @@
           <t>Purchase turnover (annualized purchase volume ÷ avg receivables)</t>
         </is>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="18">
         <f>B11*12/months/avg_rec</f>
         <v/>
       </c>
@@ -1503,7 +1621,7 @@
           <t>Interchange rate on purchase volume</t>
         </is>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="19">
         <f>B14/B11</f>
         <v/>
       </c>
@@ -1514,16 +1632,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Interchange income = rate × purchase turnover</t>
         </is>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <f>interchange</f>
         <v/>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="17">
         <f>C13*C12</f>
         <v/>
       </c>
@@ -1545,16 +1663,16 @@
       <c r="D16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Gross yield — all revenue</t>
         </is>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="16">
         <f>B8+B14</f>
         <v/>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="17">
         <f>C8+C14</f>
         <v/>
       </c>
@@ -1581,7 +1699,7 @@
           <t>Principal flow (purchase volume + pay-a-friend)</t>
         </is>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="13">
         <f>flow</f>
         <v/>
       </c>
@@ -1592,7 +1710,7 @@
           <t>Principal turnover (annualized principal flow ÷ avg receivables)</t>
         </is>
       </c>
-      <c r="C21" s="17">
+      <c r="C21" s="18">
         <f>B20*12/months/avg_rec</f>
         <v/>
       </c>
@@ -1608,7 +1726,7 @@
           <t>Loss rate — ≥90 DPD ex-FPD, vintages since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="20">
         <f>L_x90</f>
         <v/>
       </c>
@@ -1619,13 +1737,13 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Loss on receivables — ex-FPD (rate × turnover)</t>
         </is>
       </c>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="16">
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="17">
         <f>C22*C21</f>
         <v/>
       </c>
@@ -1636,7 +1754,7 @@
           <t>Loss rate — ≥90 DPD all accounts (what the tape shows before the FPD carve-out)</t>
         </is>
       </c>
-      <c r="C24" s="19">
+      <c r="C24" s="20">
         <f>L_all90</f>
         <v/>
       </c>
@@ -1647,7 +1765,7 @@
           <t>Loss on receivables — all accounts</t>
         </is>
       </c>
-      <c r="C25" s="13">
+      <c r="C25" s="14">
         <f>C24*C21</f>
         <v/>
       </c>
@@ -1658,7 +1776,7 @@
           <t xml:space="preserve">  FPD cost = difference, borne by Zed if FPD receivables are ineligible</t>
         </is>
       </c>
-      <c r="C26" s="13">
+      <c r="C26" s="14">
         <f>C25-C23</f>
         <v/>
       </c>
@@ -1693,11 +1811,11 @@
           <t>Gross yield</t>
         </is>
       </c>
-      <c r="B30" s="13">
+      <c r="B30" s="14">
         <f>C17</f>
         <v/>
       </c>
-      <c r="C30" s="13">
+      <c r="C30" s="14">
         <f>C17</f>
         <v/>
       </c>
@@ -1708,11 +1826,11 @@
           <t>− Loss on receivables</t>
         </is>
       </c>
-      <c r="B31" s="13">
+      <c r="B31" s="14">
         <f>C23</f>
         <v/>
       </c>
-      <c r="C31" s="13">
+      <c r="C31" s="14">
         <f>C25</f>
         <v/>
       </c>
@@ -1723,16 +1841,16 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>⇒ Net yield (before servicing/opex/funding)</t>
         </is>
       </c>
-      <c r="B32" s="16">
+      <c r="B32" s="17">
         <f>B30-B31</f>
         <v/>
       </c>
-      <c r="C32" s="16">
+      <c r="C32" s="17">
         <f>C30-C31</f>
         <v/>
       </c>
@@ -1743,11 +1861,11 @@
           <t>− Cost of funds on receivables = coupon × advance rate</t>
         </is>
       </c>
-      <c r="B33" s="13">
+      <c r="B33" s="14">
         <f>coupon*advance</f>
         <v/>
       </c>
-      <c r="C33" s="13">
+      <c r="C33" s="14">
         <f>coupon*advance</f>
         <v/>
       </c>
@@ -1763,11 +1881,11 @@
           <t>− Withholding gross-up (placeholder, 0)</t>
         </is>
       </c>
-      <c r="B34" s="13">
+      <c r="B34" s="14">
         <f>coupon*advance*wht/(1-wht)</f>
         <v/>
       </c>
-      <c r="C34" s="13">
+      <c r="C34" s="14">
         <f>coupon*advance*wht/(1-wht)</f>
         <v/>
       </c>
@@ -1783,26 +1901,26 @@
           <t>− FX hedge (placeholder, 0)</t>
         </is>
       </c>
-      <c r="B35" s="13">
+      <c r="B35" s="14">
         <f>hedge*advance</f>
         <v/>
       </c>
-      <c r="C35" s="13">
+      <c r="C35" s="14">
         <f>hedge*advance</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>⇒ Excess spread on receivables</t>
         </is>
       </c>
-      <c r="B36" s="16">
+      <c r="B36" s="17">
         <f>B32-B33-B34-B35</f>
         <v/>
       </c>
-      <c r="C36" s="16">
+      <c r="C36" s="17">
         <f>C32-C33-C34-C35</f>
         <v/>
       </c>
@@ -1818,11 +1936,11 @@
           <t>Excess spread on the drawn amount (÷ advance rate)</t>
         </is>
       </c>
-      <c r="B37" s="13">
+      <c r="B37" s="14">
         <f>B36/advance</f>
         <v/>
       </c>
-      <c r="C37" s="13">
+      <c r="C37" s="14">
         <f>C36/advance</f>
         <v/>
       </c>
@@ -1838,11 +1956,11 @@
           <t>Coverage = net yield ÷ cost of funds</t>
         </is>
       </c>
-      <c r="B38" s="20">
+      <c r="B38" s="21">
         <f>B32/(B33+B34+B35)</f>
         <v/>
       </c>
-      <c r="C38" s="20">
+      <c r="C38" s="21">
         <f>C32/(C33+C34+C35)</f>
         <v/>
       </c>
@@ -1858,11 +1976,11 @@
           <t>Breakeven loss rate on originations (excess spread = 0)</t>
         </is>
       </c>
-      <c r="B39" s="18">
+      <c r="B39" s="19">
         <f>(B30-B33-B34-B35)/C21</f>
         <v/>
       </c>
-      <c r="C39" s="18">
+      <c r="C39" s="19">
         <f>(C30-C33-C34-C35)/C21</f>
         <v/>
       </c>
@@ -1878,11 +1996,11 @@
           <t>Headroom: breakeven ÷ current loss rate</t>
         </is>
       </c>
-      <c r="B40" s="20">
+      <c r="B40" s="21">
         <f>B39/C22</f>
         <v/>
       </c>
-      <c r="C40" s="20">
+      <c r="C40" s="21">
         <f>C39/C24</f>
         <v/>
       </c>
@@ -1898,11 +2016,11 @@
           <t>Return on Zed's unfunded slice = excess spread ÷ (1 − advance), before opex</t>
         </is>
       </c>
-      <c r="B41" s="13">
+      <c r="B41" s="14">
         <f>B36/(1-advance)</f>
         <v/>
       </c>
-      <c r="C41" s="13">
+      <c r="C41" s="14">
         <f>C36/(1-advance)</f>
         <v/>
       </c>
@@ -1914,7 +2032,7 @@
     </row>
     <row r="42"/>
     <row r="43" ht="48" customHeight="1">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>Read: the lender underwrites the left column (its pool excludes FPD receivables, which Zed repurchases); Zed lives in the right column. Today the FPD cost (row 26) consumes nearly all of Zed's excess spread — the new fraud controls are the margin. Frictions (withholding, hedge) are placeholders at 0 and would come off Zed's column.</t>
         </is>
@@ -1934,7 +2052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
@@ -1956,7 +2074,7 @@
       </c>
     </row>
     <row r="2" ht="64" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Model: transacting and installment balances held at Q3 levels; revolving balance scaled to hit the target share of balances; revolving interest = Q3 monthly rate × 12 on the revolving balance; purchase volume, pay-a-friend, interchange, installment charges and late fees held in pesos (spend- and conversion-driven, not balance-driven); principal flow therefore held, so turnover falls as the book grows and the same loss rate on originations becomes a smaller loss on balances. Cost of funds = coupon × advance rate; withholding and hedge at their Inputs values (0 unless set).</t>
         </is>
@@ -1981,1298 +2099,1402 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Revolving monthly rate on revolving balance</t>
-        </is>
-      </c>
-      <c r="B5" s="18">
-        <f>rev_int/(bal_rev*months)</f>
-        <v/>
-      </c>
-      <c r="C5" s="23" t="inlineStr">
-        <is>
-          <t>rev_int ÷ Σ monthly revolving balances (Jul–Sep) — 2.44%; BSP cap 3%</t>
+          <t>Monthly rate on the interest-bearing balance (3.05%; 36.5% APR)</t>
+        </is>
+      </c>
+      <c r="B5" s="19">
+        <f>rate_ib</f>
+        <v/>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>rev_int ÷ Σ purchase_interest_balance on revolver statements, Jul–Sep</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Revolving share of balances, Q3 average</t>
-        </is>
-      </c>
-      <c r="B6" s="13">
-        <f>bal_rev/bal_tot</f>
-        <v/>
+          <t>Interest-bearing balance ÷ revolving-bucket balance (scenario)</t>
+        </is>
+      </c>
+      <c r="B6" s="25">
+        <f>ratio_scn</f>
+        <v/>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>observed 0.80 in Q3 (growth/timing); effective yield on the bucket = rate × ratio = 2.44%/month</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Non-revolving balance (transacting + installment), scaled to avg receivables</t>
-        </is>
-      </c>
-      <c r="B7" s="12">
-        <f>(bal_tra+bal_inst)/bal_tot*avg_rec</f>
-        <v/>
-      </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>held constant across scenarios</t>
-        </is>
+          <t>Revolving share of balances, Q3 average</t>
+        </is>
+      </c>
+      <c r="B7" s="14">
+        <f>bal_rev/bal_tot</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Annual principal flow (Q3 × 4)</t>
-        </is>
-      </c>
-      <c r="B8" s="12">
-        <f>flow*12/months</f>
-        <v/>
-      </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>held constant</t>
+          <t>Non-revolving balance (transacting + installment), scaled to avg receivables</t>
+        </is>
+      </c>
+      <c r="B8" s="13">
+        <f>(bal_tra+bal_inst)/bal_tot*avg_rec</f>
+        <v/>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>held constant across scenarios</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Annual interchange + installment charges + late fees (Q3 × 4)</t>
-        </is>
-      </c>
-      <c r="B9" s="12">
-        <f>(interchange+inst_int+upfront+late)*12/months</f>
-        <v/>
-      </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>held constant in pesos</t>
+          <t>Annual principal flow (Q3 × 4)</t>
+        </is>
+      </c>
+      <c r="B9" s="13">
+        <f>flow*12/months</f>
+        <v/>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>held constant</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Annual interchange + installment charges + late fees (Q3 × 4)</t>
+        </is>
+      </c>
+      <c r="B10" s="13">
+        <f>(interchange+inst_int+upfront+late)*12/months</f>
+        <v/>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>held constant in pesos</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Friction add-on to cost of funds (withholding gross-up + hedge), pts of receivables</t>
         </is>
       </c>
-      <c r="B10" s="18">
+      <c r="B11" s="19">
         <f>coupon*advance*wht/(1-wht)+hedge*advance</f>
         <v/>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>0 unless set on Inputs</t>
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Revolving share of balances = Q3 average</t>
         </is>
       </c>
-      <c r="B12" s="24">
+      <c r="B13" s="26">
         <f>bal_rev/bal_tot</f>
         <v/>
       </c>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Revolving balance (PHP)</t>
-        </is>
-      </c>
-      <c r="B13" s="12">
-        <f>$B$12/(1-$B$12)*$B$7</f>
-        <v/>
-      </c>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Total receivables (PHP)</t>
-        </is>
-      </c>
-      <c r="B14" s="12">
-        <f>$B$7+B13</f>
+          <t>Revolving balance (PHP)</t>
+        </is>
+      </c>
+      <c r="B14" s="13">
+        <f>$B$13/(1-$B$13)*s_nonrev</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gross yield — all revenue</t>
+          <t>Total receivables (PHP)</t>
         </is>
       </c>
       <c r="B15" s="13">
-        <f>($B$5*12*B13+$B$9)/B14</f>
+        <f>s_nonrev+B14</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  of which interest and fees</t>
-        </is>
-      </c>
-      <c r="B16" s="13">
-        <f>($B$5*12*B13+(inst_int+upfront+late)*12/months)/B14</f>
+          <t>Gross yield — all revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="14">
+        <f>(s_rate*s_ratio*12*B14+s_other)/B15</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t xml:space="preserve">  of which interest and fees</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>(s_rate*s_ratio*12*B14+(inst_int+upfront+late)*12/months)/B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Principal turnover (x per year)</t>
         </is>
       </c>
-      <c r="B17" s="17">
-        <f>$B$8/B14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="B18" s="18">
+        <f>s_flow/B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Excess spread, pts of receivables — coupon ↓ / loss rate →</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C19" s="25" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
       </c>
-      <c r="D19" s="25" t="inlineStr">
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E19" s="25" t="inlineStr">
+      <c r="E20" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
       </c>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="G20" s="15" t="inlineStr">
         <is>
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H19" s="25" t="inlineStr">
+      <c r="H20" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I19" s="25" t="inlineStr">
+      <c r="I20" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
-        </is>
-      </c>
-      <c r="B20" s="13">
-        <f>$B$15-L_x90*$B$17-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C20" s="13">
-        <f>$B$15-L_all90*$B$17-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D20" s="13">
-        <f>$B$15-L_life90x*$B$17-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E20" s="13">
-        <f>$B$15-L_life90*$B$17-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H20" s="13">
-        <f>$B$15-L_x90*$B$17</f>
-        <v/>
-      </c>
-      <c r="I20" s="13">
-        <f>$B$15-L_all90*$B$17</f>
-        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
-        </is>
-      </c>
-      <c r="B21" s="13">
-        <f>$B$15-L_x90*$B$17-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C21" s="13">
-        <f>$B$15-L_all90*$B$17-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D21" s="13">
-        <f>$B$15-L_life90x*$B$17-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E21" s="13">
-        <f>$B$15-L_life90*$B$17-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H21" s="13">
-        <f>$B$15-L_x90*$B$17</f>
-        <v/>
-      </c>
-      <c r="I21" s="13">
-        <f>$B$15-L_all90*$B$17</f>
+          <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
+        </is>
+      </c>
+      <c r="B21" s="14">
+        <f>$B$16-L_x90*$B$18-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C21" s="14">
+        <f>$B$16-L_all90*$B$18-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D21" s="14">
+        <f>$B$16-L_life90x*$B$18-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E21" s="14">
+        <f>$B$16-L_life90*$B$18-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H21" s="14">
+        <f>$B$16-L_x90*$B$18</f>
+        <v/>
+      </c>
+      <c r="I21" s="14">
+        <f>$B$16-L_all90*$B$18</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
+        </is>
+      </c>
+      <c r="B22" s="14">
+        <f>$B$16-L_x90*$B$18-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C22" s="14">
+        <f>$B$16-L_all90*$B$18-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D22" s="14">
+        <f>$B$16-L_life90x*$B$18-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E22" s="14">
+        <f>$B$16-L_life90*$B$18-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H22" s="14">
+        <f>$B$16-L_x90*$B$18</f>
+        <v/>
+      </c>
+      <c r="I22" s="14">
+        <f>$B$16-L_all90*$B$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Coupon 19% (cost on receivables = 19% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B22" s="13">
-        <f>$B$15-L_x90*$B$17-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C22" s="13">
-        <f>$B$15-L_all90*$B$17-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D22" s="13">
-        <f>$B$15-L_life90x*$B$17-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E22" s="13">
-        <f>$B$15-L_life90*$B$17-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H22" s="13">
-        <f>$B$15-L_x90*$B$17</f>
-        <v/>
-      </c>
-      <c r="I22" s="13">
-        <f>$B$15-L_all90*$B$17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="B23" s="14">
+        <f>$B$16-L_x90*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C23" s="14">
+        <f>$B$16-L_all90*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D23" s="14">
+        <f>$B$16-L_life90x*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E23" s="14">
+        <f>$B$16-L_life90*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H23" s="14">
+        <f>$B$16-L_x90*$B$18</f>
+        <v/>
+      </c>
+      <c r="I23" s="14">
+        <f>$B$16-L_all90*$B$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Advance rate sensitivity at 19% coupon, base loss — advance →</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B25" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="C24" s="16" t="n">
+      <c r="C25" s="17" t="n">
         <v>0.75</v>
       </c>
-      <c r="D24" s="16" t="n">
+      <c r="D25" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="E24" s="16" t="n">
+      <c r="E25" s="17" t="n">
         <v>0.85</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Excess spread, pts of receivables</t>
-        </is>
-      </c>
-      <c r="B25" s="13">
-        <f>$B$15-L_x90*$B$17-0.19*B24-$B$10</f>
-        <v/>
-      </c>
-      <c r="C25" s="13">
-        <f>$B$15-L_x90*$B$17-0.19*C24-$B$10</f>
-        <v/>
-      </c>
-      <c r="D25" s="13">
-        <f>$B$15-L_x90*$B$17-0.19*D24-$B$10</f>
-        <v/>
-      </c>
-      <c r="E25" s="13">
-        <f>$B$15-L_x90*$B$17-0.19*E24-$B$10</f>
-        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
-        </is>
-      </c>
-      <c r="B26" s="20">
-        <f>($B$15-L_x90*$B$17)/(0.19*B24+$B$10)</f>
-        <v/>
-      </c>
-      <c r="C26" s="20">
-        <f>($B$15-L_x90*$B$17)/(0.19*C24+$B$10)</f>
-        <v/>
-      </c>
-      <c r="D26" s="20">
-        <f>($B$15-L_x90*$B$17)/(0.19*D24+$B$10)</f>
-        <v/>
-      </c>
-      <c r="E26" s="20">
-        <f>($B$15-L_x90*$B$17)/(0.19*E24+$B$10)</f>
+          <t xml:space="preserve">  Excess spread, pts of receivables</t>
+        </is>
+      </c>
+      <c r="B26" s="14">
+        <f>$B$16-L_x90*$B$18-0.19*B25-s_fric</f>
+        <v/>
+      </c>
+      <c r="C26" s="14">
+        <f>$B$16-L_x90*$B$18-0.19*C25-s_fric</f>
+        <v/>
+      </c>
+      <c r="D26" s="14">
+        <f>$B$16-L_x90*$B$18-0.19*D25-s_fric</f>
+        <v/>
+      </c>
+      <c r="E26" s="14">
+        <f>$B$16-L_x90*$B$18-0.19*E25-s_fric</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
+        </is>
+      </c>
+      <c r="B27" s="21">
+        <f>($B$16-L_x90*$B$18)/(0.19*B25+s_fric)</f>
+        <v/>
+      </c>
+      <c r="C27" s="21">
+        <f>($B$16-L_x90*$B$18)/(0.19*C25+s_fric)</f>
+        <v/>
+      </c>
+      <c r="D27" s="21">
+        <f>($B$16-L_x90*$B$18)/(0.19*D25+s_fric)</f>
+        <v/>
+      </c>
+      <c r="E27" s="21">
+        <f>($B$16-L_x90*$B$18)/(0.19*E25+s_fric)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Breakeven loss rate on originations</t>
         </is>
       </c>
-      <c r="B27" s="18">
-        <f>($B$15-0.19*B24-$B$10)/$B$17</f>
-        <v/>
-      </c>
-      <c r="C27" s="18">
-        <f>($B$15-0.19*C24-$B$10)/$B$17</f>
-        <v/>
-      </c>
-      <c r="D27" s="18">
-        <f>($B$15-0.19*D24-$B$10)/$B$17</f>
-        <v/>
-      </c>
-      <c r="E27" s="18">
-        <f>($B$15-0.19*E24-$B$10)/$B$17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="B28" s="19">
+        <f>($B$16-0.19*B25-s_fric)/$B$18</f>
+        <v/>
+      </c>
+      <c r="C28" s="19">
+        <f>($B$16-0.19*C25-s_fric)/$B$18</f>
+        <v/>
+      </c>
+      <c r="D28" s="19">
+        <f>($B$16-0.19*D25-s_fric)/$B$18</f>
+        <v/>
+      </c>
+      <c r="E28" s="19">
+        <f>($B$16-0.19*E25-s_fric)/$B$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Revolving share of balances = 50%</t>
         </is>
       </c>
-      <c r="B29" s="24" t="n">
+      <c r="B30" s="26" t="n">
         <v>0.5</v>
       </c>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="n"/>
-      <c r="I29" s="5" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Revolving balance (PHP)</t>
-        </is>
-      </c>
-      <c r="B30" s="12">
-        <f>$B$29/(1-$B$29)*$B$7</f>
-        <v/>
-      </c>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Total receivables (PHP)</t>
-        </is>
-      </c>
-      <c r="B31" s="12">
-        <f>$B$7+B30</f>
+          <t>Revolving balance (PHP)</t>
+        </is>
+      </c>
+      <c r="B31" s="13">
+        <f>$B$30/(1-$B$30)*s_nonrev</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Gross yield — all revenue</t>
+          <t>Total receivables (PHP)</t>
         </is>
       </c>
       <c r="B32" s="13">
-        <f>($B$5*12*B30+$B$9)/B31</f>
+        <f>s_nonrev+B31</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  of which interest and fees</t>
-        </is>
-      </c>
-      <c r="B33" s="13">
-        <f>($B$5*12*B30+(inst_int+upfront+late)*12/months)/B31</f>
+          <t>Gross yield — all revenue</t>
+        </is>
+      </c>
+      <c r="B33" s="14">
+        <f>(s_rate*s_ratio*12*B31+s_other)/B32</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t xml:space="preserve">  of which interest and fees</t>
+        </is>
+      </c>
+      <c r="B34" s="14">
+        <f>(s_rate*s_ratio*12*B31+(inst_int+upfront+late)*12/months)/B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Principal turnover (x per year)</t>
         </is>
       </c>
-      <c r="B34" s="17">
-        <f>$B$8/B31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35"/>
-    <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="B35" s="18">
+        <f>s_flow/B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>Excess spread, pts of receivables — coupon ↓ / loss rate →</t>
         </is>
       </c>
-      <c r="B36" s="25" t="inlineStr">
+      <c r="B37" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C36" s="25" t="inlineStr">
+      <c r="C37" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
       </c>
-      <c r="D36" s="25" t="inlineStr">
+      <c r="D37" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E36" s="25" t="inlineStr">
+      <c r="E37" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
+      <c r="G37" s="15" t="inlineStr">
         <is>
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H36" s="25" t="inlineStr">
+      <c r="H37" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I36" s="25" t="inlineStr">
+      <c r="I37" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
-        </is>
-      </c>
-      <c r="B37" s="13">
-        <f>$B$32-L_x90*$B$34-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C37" s="13">
-        <f>$B$32-L_all90*$B$34-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D37" s="13">
-        <f>$B$32-L_life90x*$B$34-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E37" s="13">
-        <f>$B$32-L_life90*$B$34-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H37" s="13">
-        <f>$B$32-L_x90*$B$34</f>
-        <v/>
-      </c>
-      <c r="I37" s="13">
-        <f>$B$32-L_all90*$B$34</f>
-        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
-        </is>
-      </c>
-      <c r="B38" s="13">
-        <f>$B$32-L_x90*$B$34-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C38" s="13">
-        <f>$B$32-L_all90*$B$34-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D38" s="13">
-        <f>$B$32-L_life90x*$B$34-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E38" s="13">
-        <f>$B$32-L_life90*$B$34-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H38" s="13">
-        <f>$B$32-L_x90*$B$34</f>
-        <v/>
-      </c>
-      <c r="I38" s="13">
-        <f>$B$32-L_all90*$B$34</f>
+          <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
+        </is>
+      </c>
+      <c r="B38" s="14">
+        <f>$B$33-L_x90*$B$35-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C38" s="14">
+        <f>$B$33-L_all90*$B$35-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D38" s="14">
+        <f>$B$33-L_life90x*$B$35-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E38" s="14">
+        <f>$B$33-L_life90*$B$35-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H38" s="14">
+        <f>$B$33-L_x90*$B$35</f>
+        <v/>
+      </c>
+      <c r="I38" s="14">
+        <f>$B$33-L_all90*$B$35</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
+        </is>
+      </c>
+      <c r="B39" s="14">
+        <f>$B$33-L_x90*$B$35-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C39" s="14">
+        <f>$B$33-L_all90*$B$35-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D39" s="14">
+        <f>$B$33-L_life90x*$B$35-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E39" s="14">
+        <f>$B$33-L_life90*$B$35-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H39" s="14">
+        <f>$B$33-L_x90*$B$35</f>
+        <v/>
+      </c>
+      <c r="I39" s="14">
+        <f>$B$33-L_all90*$B$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>Coupon 19% (cost on receivables = 19% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B39" s="13">
-        <f>$B$32-L_x90*$B$34-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C39" s="13">
-        <f>$B$32-L_all90*$B$34-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D39" s="13">
-        <f>$B$32-L_life90x*$B$34-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E39" s="13">
-        <f>$B$32-L_life90*$B$34-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H39" s="13">
-        <f>$B$32-L_x90*$B$34</f>
-        <v/>
-      </c>
-      <c r="I39" s="13">
-        <f>$B$32-L_all90*$B$34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="B40" s="14">
+        <f>$B$33-L_x90*$B$35-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C40" s="14">
+        <f>$B$33-L_all90*$B$35-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D40" s="14">
+        <f>$B$33-L_life90x*$B$35-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E40" s="14">
+        <f>$B$33-L_life90*$B$35-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H40" s="14">
+        <f>$B$33-L_x90*$B$35</f>
+        <v/>
+      </c>
+      <c r="I40" s="14">
+        <f>$B$33-L_all90*$B$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>Advance rate sensitivity at 19% coupon, base loss — advance →</t>
         </is>
       </c>
-      <c r="B41" s="16" t="n">
+      <c r="B42" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="C41" s="16" t="n">
+      <c r="C42" s="17" t="n">
         <v>0.75</v>
       </c>
-      <c r="D41" s="16" t="n">
+      <c r="D42" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="E41" s="16" t="n">
+      <c r="E42" s="17" t="n">
         <v>0.85</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Excess spread, pts of receivables</t>
-        </is>
-      </c>
-      <c r="B42" s="13">
-        <f>$B$32-L_x90*$B$34-0.19*B41-$B$10</f>
-        <v/>
-      </c>
-      <c r="C42" s="13">
-        <f>$B$32-L_x90*$B$34-0.19*C41-$B$10</f>
-        <v/>
-      </c>
-      <c r="D42" s="13">
-        <f>$B$32-L_x90*$B$34-0.19*D41-$B$10</f>
-        <v/>
-      </c>
-      <c r="E42" s="13">
-        <f>$B$32-L_x90*$B$34-0.19*E41-$B$10</f>
-        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
-        </is>
-      </c>
-      <c r="B43" s="20">
-        <f>($B$32-L_x90*$B$34)/(0.19*B41+$B$10)</f>
-        <v/>
-      </c>
-      <c r="C43" s="20">
-        <f>($B$32-L_x90*$B$34)/(0.19*C41+$B$10)</f>
-        <v/>
-      </c>
-      <c r="D43" s="20">
-        <f>($B$32-L_x90*$B$34)/(0.19*D41+$B$10)</f>
-        <v/>
-      </c>
-      <c r="E43" s="20">
-        <f>($B$32-L_x90*$B$34)/(0.19*E41+$B$10)</f>
+          <t xml:space="preserve">  Excess spread, pts of receivables</t>
+        </is>
+      </c>
+      <c r="B43" s="14">
+        <f>$B$33-L_x90*$B$35-0.19*B42-s_fric</f>
+        <v/>
+      </c>
+      <c r="C43" s="14">
+        <f>$B$33-L_x90*$B$35-0.19*C42-s_fric</f>
+        <v/>
+      </c>
+      <c r="D43" s="14">
+        <f>$B$33-L_x90*$B$35-0.19*D42-s_fric</f>
+        <v/>
+      </c>
+      <c r="E43" s="14">
+        <f>$B$33-L_x90*$B$35-0.19*E42-s_fric</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
+        </is>
+      </c>
+      <c r="B44" s="21">
+        <f>($B$33-L_x90*$B$35)/(0.19*B42+s_fric)</f>
+        <v/>
+      </c>
+      <c r="C44" s="21">
+        <f>($B$33-L_x90*$B$35)/(0.19*C42+s_fric)</f>
+        <v/>
+      </c>
+      <c r="D44" s="21">
+        <f>($B$33-L_x90*$B$35)/(0.19*D42+s_fric)</f>
+        <v/>
+      </c>
+      <c r="E44" s="21">
+        <f>($B$33-L_x90*$B$35)/(0.19*E42+s_fric)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Breakeven loss rate on originations</t>
         </is>
       </c>
-      <c r="B44" s="18">
-        <f>($B$32-0.19*B41-$B$10)/$B$34</f>
-        <v/>
-      </c>
-      <c r="C44" s="18">
-        <f>($B$32-0.19*C41-$B$10)/$B$34</f>
-        <v/>
-      </c>
-      <c r="D44" s="18">
-        <f>($B$32-0.19*D41-$B$10)/$B$34</f>
-        <v/>
-      </c>
-      <c r="E44" s="18">
-        <f>($B$32-0.19*E41-$B$10)/$B$34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45"/>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="B45" s="19">
+        <f>($B$33-0.19*B42-s_fric)/$B$35</f>
+        <v/>
+      </c>
+      <c r="C45" s="19">
+        <f>($B$33-0.19*C42-s_fric)/$B$35</f>
+        <v/>
+      </c>
+      <c r="D45" s="19">
+        <f>($B$33-0.19*D42-s_fric)/$B$35</f>
+        <v/>
+      </c>
+      <c r="E45" s="19">
+        <f>($B$33-0.19*E42-s_fric)/$B$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>Revolving share of balances = 55%</t>
         </is>
       </c>
-      <c r="B46" s="24" t="n">
+      <c r="B47" s="26" t="n">
         <v>0.55</v>
       </c>
-      <c r="C46" s="5" t="n"/>
-      <c r="D46" s="5" t="n"/>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46" s="5" t="n"/>
-      <c r="G46" s="5" t="n"/>
-      <c r="H46" s="5" t="n"/>
-      <c r="I46" s="5" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Revolving balance (PHP)</t>
-        </is>
-      </c>
-      <c r="B47" s="12">
-        <f>$B$46/(1-$B$46)*$B$7</f>
-        <v/>
-      </c>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Total receivables (PHP)</t>
-        </is>
-      </c>
-      <c r="B48" s="12">
-        <f>$B$7+B47</f>
+          <t>Revolving balance (PHP)</t>
+        </is>
+      </c>
+      <c r="B48" s="13">
+        <f>$B$47/(1-$B$47)*s_nonrev</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Gross yield — all revenue</t>
+          <t>Total receivables (PHP)</t>
         </is>
       </c>
       <c r="B49" s="13">
-        <f>($B$5*12*B47+$B$9)/B48</f>
+        <f>s_nonrev+B48</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  of which interest and fees</t>
-        </is>
-      </c>
-      <c r="B50" s="13">
-        <f>($B$5*12*B47+(inst_int+upfront+late)*12/months)/B48</f>
+          <t>Gross yield — all revenue</t>
+        </is>
+      </c>
+      <c r="B50" s="14">
+        <f>(s_rate*s_ratio*12*B48+s_other)/B49</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t xml:space="preserve">  of which interest and fees</t>
+        </is>
+      </c>
+      <c r="B51" s="14">
+        <f>(s_rate*s_ratio*12*B48+(inst_int+upfront+late)*12/months)/B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>Principal turnover (x per year)</t>
         </is>
       </c>
-      <c r="B51" s="17">
-        <f>$B$8/B48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52"/>
-    <row r="53" ht="32" customHeight="1">
-      <c r="A53" s="14" t="inlineStr">
+      <c r="B52" s="18">
+        <f>s_flow/B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53"/>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>Excess spread, pts of receivables — coupon ↓ / loss rate →</t>
         </is>
       </c>
-      <c r="B53" s="25" t="inlineStr">
+      <c r="B54" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C53" s="25" t="inlineStr">
+      <c r="C54" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
       </c>
-      <c r="D53" s="25" t="inlineStr">
+      <c r="D54" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E53" s="25" t="inlineStr">
+      <c r="E54" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
       </c>
-      <c r="G53" s="14" t="inlineStr">
+      <c r="G54" s="15" t="inlineStr">
         <is>
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H53" s="25" t="inlineStr">
+      <c r="H54" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I53" s="25" t="inlineStr">
+      <c r="I54" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
-        </is>
-      </c>
-      <c r="B54" s="13">
-        <f>$B$49-L_x90*$B$51-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C54" s="13">
-        <f>$B$49-L_all90*$B$51-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D54" s="13">
-        <f>$B$49-L_life90x*$B$51-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E54" s="13">
-        <f>$B$49-L_life90*$B$51-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H54" s="13">
-        <f>$B$49-L_x90*$B$51</f>
-        <v/>
-      </c>
-      <c r="I54" s="13">
-        <f>$B$49-L_all90*$B$51</f>
-        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
-        </is>
-      </c>
-      <c r="B55" s="13">
-        <f>$B$49-L_x90*$B$51-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C55" s="13">
-        <f>$B$49-L_all90*$B$51-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D55" s="13">
-        <f>$B$49-L_life90x*$B$51-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E55" s="13">
-        <f>$B$49-L_life90*$B$51-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H55" s="13">
-        <f>$B$49-L_x90*$B$51</f>
-        <v/>
-      </c>
-      <c r="I55" s="13">
-        <f>$B$49-L_all90*$B$51</f>
+          <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
+        </is>
+      </c>
+      <c r="B55" s="14">
+        <f>$B$50-L_x90*$B$52-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C55" s="14">
+        <f>$B$50-L_all90*$B$52-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D55" s="14">
+        <f>$B$50-L_life90x*$B$52-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E55" s="14">
+        <f>$B$50-L_life90*$B$52-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H55" s="14">
+        <f>$B$50-L_x90*$B$52</f>
+        <v/>
+      </c>
+      <c r="I55" s="14">
+        <f>$B$50-L_all90*$B$52</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
+        </is>
+      </c>
+      <c r="B56" s="14">
+        <f>$B$50-L_x90*$B$52-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C56" s="14">
+        <f>$B$50-L_all90*$B$52-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D56" s="14">
+        <f>$B$50-L_life90x*$B$52-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E56" s="14">
+        <f>$B$50-L_life90*$B$52-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H56" s="14">
+        <f>$B$50-L_x90*$B$52</f>
+        <v/>
+      </c>
+      <c r="I56" s="14">
+        <f>$B$50-L_all90*$B$52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>Coupon 19% (cost on receivables = 19% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B56" s="13">
-        <f>$B$49-L_x90*$B$51-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C56" s="13">
-        <f>$B$49-L_all90*$B$51-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D56" s="13">
-        <f>$B$49-L_life90x*$B$51-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E56" s="13">
-        <f>$B$49-L_life90*$B$51-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H56" s="13">
-        <f>$B$49-L_x90*$B$51</f>
-        <v/>
-      </c>
-      <c r="I56" s="13">
-        <f>$B$49-L_all90*$B$51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57"/>
-    <row r="58">
-      <c r="A58" s="14" t="inlineStr">
+      <c r="B57" s="14">
+        <f>$B$50-L_x90*$B$52-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C57" s="14">
+        <f>$B$50-L_all90*$B$52-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D57" s="14">
+        <f>$B$50-L_life90x*$B$52-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E57" s="14">
+        <f>$B$50-L_life90*$B$52-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H57" s="14">
+        <f>$B$50-L_x90*$B$52</f>
+        <v/>
+      </c>
+      <c r="I57" s="14">
+        <f>$B$50-L_all90*$B$52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58"/>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>Advance rate sensitivity at 19% coupon, base loss — advance →</t>
         </is>
       </c>
-      <c r="B58" s="16" t="n">
+      <c r="B59" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="C58" s="16" t="n">
+      <c r="C59" s="17" t="n">
         <v>0.75</v>
       </c>
-      <c r="D58" s="16" t="n">
+      <c r="D59" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="E58" s="16" t="n">
+      <c r="E59" s="17" t="n">
         <v>0.85</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Excess spread, pts of receivables</t>
-        </is>
-      </c>
-      <c r="B59" s="13">
-        <f>$B$49-L_x90*$B$51-0.19*B58-$B$10</f>
-        <v/>
-      </c>
-      <c r="C59" s="13">
-        <f>$B$49-L_x90*$B$51-0.19*C58-$B$10</f>
-        <v/>
-      </c>
-      <c r="D59" s="13">
-        <f>$B$49-L_x90*$B$51-0.19*D58-$B$10</f>
-        <v/>
-      </c>
-      <c r="E59" s="13">
-        <f>$B$49-L_x90*$B$51-0.19*E58-$B$10</f>
-        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
-        </is>
-      </c>
-      <c r="B60" s="20">
-        <f>($B$49-L_x90*$B$51)/(0.19*B58+$B$10)</f>
-        <v/>
-      </c>
-      <c r="C60" s="20">
-        <f>($B$49-L_x90*$B$51)/(0.19*C58+$B$10)</f>
-        <v/>
-      </c>
-      <c r="D60" s="20">
-        <f>($B$49-L_x90*$B$51)/(0.19*D58+$B$10)</f>
-        <v/>
-      </c>
-      <c r="E60" s="20">
-        <f>($B$49-L_x90*$B$51)/(0.19*E58+$B$10)</f>
+          <t xml:space="preserve">  Excess spread, pts of receivables</t>
+        </is>
+      </c>
+      <c r="B60" s="14">
+        <f>$B$50-L_x90*$B$52-0.19*B59-s_fric</f>
+        <v/>
+      </c>
+      <c r="C60" s="14">
+        <f>$B$50-L_x90*$B$52-0.19*C59-s_fric</f>
+        <v/>
+      </c>
+      <c r="D60" s="14">
+        <f>$B$50-L_x90*$B$52-0.19*D59-s_fric</f>
+        <v/>
+      </c>
+      <c r="E60" s="14">
+        <f>$B$50-L_x90*$B$52-0.19*E59-s_fric</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
+        </is>
+      </c>
+      <c r="B61" s="21">
+        <f>($B$50-L_x90*$B$52)/(0.19*B59+s_fric)</f>
+        <v/>
+      </c>
+      <c r="C61" s="21">
+        <f>($B$50-L_x90*$B$52)/(0.19*C59+s_fric)</f>
+        <v/>
+      </c>
+      <c r="D61" s="21">
+        <f>($B$50-L_x90*$B$52)/(0.19*D59+s_fric)</f>
+        <v/>
+      </c>
+      <c r="E61" s="21">
+        <f>($B$50-L_x90*$B$52)/(0.19*E59+s_fric)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Breakeven loss rate on originations</t>
         </is>
       </c>
-      <c r="B61" s="18">
-        <f>($B$49-0.19*B58-$B$10)/$B$51</f>
-        <v/>
-      </c>
-      <c r="C61" s="18">
-        <f>($B$49-0.19*C58-$B$10)/$B$51</f>
-        <v/>
-      </c>
-      <c r="D61" s="18">
-        <f>($B$49-0.19*D58-$B$10)/$B$51</f>
-        <v/>
-      </c>
-      <c r="E61" s="18">
-        <f>($B$49-0.19*E58-$B$10)/$B$51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62"/>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+      <c r="B62" s="19">
+        <f>($B$50-0.19*B59-s_fric)/$B$52</f>
+        <v/>
+      </c>
+      <c r="C62" s="19">
+        <f>($B$50-0.19*C59-s_fric)/$B$52</f>
+        <v/>
+      </c>
+      <c r="D62" s="19">
+        <f>($B$50-0.19*D59-s_fric)/$B$52</f>
+        <v/>
+      </c>
+      <c r="E62" s="19">
+        <f>($B$50-0.19*E59-s_fric)/$B$52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63"/>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>Revolving share of balances = 60%</t>
         </is>
       </c>
-      <c r="B63" s="24" t="n">
+      <c r="B64" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="C63" s="5" t="n"/>
-      <c r="D63" s="5" t="n"/>
-      <c r="E63" s="5" t="n"/>
-      <c r="F63" s="5" t="n"/>
-      <c r="G63" s="5" t="n"/>
-      <c r="H63" s="5" t="n"/>
-      <c r="I63" s="5" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Revolving balance (PHP)</t>
-        </is>
-      </c>
-      <c r="B64" s="12">
-        <f>$B$63/(1-$B$63)*$B$7</f>
-        <v/>
-      </c>
+      <c r="C64" s="5" t="n"/>
+      <c r="D64" s="5" t="n"/>
+      <c r="E64" s="5" t="n"/>
+      <c r="F64" s="5" t="n"/>
+      <c r="G64" s="5" t="n"/>
+      <c r="H64" s="5" t="n"/>
+      <c r="I64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Total receivables (PHP)</t>
-        </is>
-      </c>
-      <c r="B65" s="12">
-        <f>$B$7+B64</f>
+          <t>Revolving balance (PHP)</t>
+        </is>
+      </c>
+      <c r="B65" s="13">
+        <f>$B$64/(1-$B$64)*s_nonrev</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Gross yield — all revenue</t>
+          <t>Total receivables (PHP)</t>
         </is>
       </c>
       <c r="B66" s="13">
-        <f>($B$5*12*B64+$B$9)/B65</f>
+        <f>s_nonrev+B65</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  of which interest and fees</t>
-        </is>
-      </c>
-      <c r="B67" s="13">
-        <f>($B$5*12*B64+(inst_int+upfront+late)*12/months)/B65</f>
+          <t>Gross yield — all revenue</t>
+        </is>
+      </c>
+      <c r="B67" s="14">
+        <f>(s_rate*s_ratio*12*B65+s_other)/B66</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t xml:space="preserve">  of which interest and fees</t>
+        </is>
+      </c>
+      <c r="B68" s="14">
+        <f>(s_rate*s_ratio*12*B65+(inst_int+upfront+late)*12/months)/B66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>Principal turnover (x per year)</t>
         </is>
       </c>
-      <c r="B68" s="17">
-        <f>$B$8/B65</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69"/>
-    <row r="70" ht="32" customHeight="1">
-      <c r="A70" s="14" t="inlineStr">
+      <c r="B69" s="18">
+        <f>s_flow/B66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70"/>
+    <row r="71" ht="32" customHeight="1">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t>Excess spread, pts of receivables — coupon ↓ / loss rate →</t>
         </is>
       </c>
-      <c r="B70" s="25" t="inlineStr">
+      <c r="B71" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="C70" s="25" t="inlineStr">
+      <c r="C71" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
       </c>
-      <c r="D70" s="25" t="inlineStr">
+      <c r="D71" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E70" s="25" t="inlineStr">
+      <c r="E71" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
       </c>
-      <c r="G70" s="14" t="inlineStr">
+      <c r="G71" s="15" t="inlineStr">
         <is>
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H70" s="25" t="inlineStr">
+      <c r="H71" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I70" s="25" t="inlineStr">
+      <c r="I71" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
         </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
-        </is>
-      </c>
-      <c r="B71" s="13">
-        <f>$B$66-L_x90*$B$68-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C71" s="13">
-        <f>$B$66-L_all90*$B$68-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D71" s="13">
-        <f>$B$66-L_life90x*$B$68-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E71" s="13">
-        <f>$B$66-L_life90*$B$68-0.15*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H71" s="13">
-        <f>$B$66-L_x90*$B$68</f>
-        <v/>
-      </c>
-      <c r="I71" s="13">
-        <f>$B$66-L_all90*$B$68</f>
-        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
-        </is>
-      </c>
-      <c r="B72" s="13">
-        <f>$B$66-L_x90*$B$68-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C72" s="13">
-        <f>$B$66-L_all90*$B$68-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D72" s="13">
-        <f>$B$66-L_life90x*$B$68-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E72" s="13">
-        <f>$B$66-L_life90*$B$68-0.17*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H72" s="13">
-        <f>$B$66-L_x90*$B$68</f>
-        <v/>
-      </c>
-      <c r="I72" s="13">
-        <f>$B$66-L_all90*$B$68</f>
+          <t>Coupon 15% (cost on receivables = 15% × advance + frictions)</t>
+        </is>
+      </c>
+      <c r="B72" s="14">
+        <f>$B$67-L_x90*$B$69-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C72" s="14">
+        <f>$B$67-L_all90*$B$69-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D72" s="14">
+        <f>$B$67-L_life90x*$B$69-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E72" s="14">
+        <f>$B$67-L_life90*$B$69-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H72" s="14">
+        <f>$B$67-L_x90*$B$69</f>
+        <v/>
+      </c>
+      <c r="I72" s="14">
+        <f>$B$67-L_all90*$B$69</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>Coupon 17% (cost on receivables = 17% × advance + frictions)</t>
+        </is>
+      </c>
+      <c r="B73" s="14">
+        <f>$B$67-L_x90*$B$69-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C73" s="14">
+        <f>$B$67-L_all90*$B$69-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D73" s="14">
+        <f>$B$67-L_life90x*$B$69-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E73" s="14">
+        <f>$B$67-L_life90*$B$69-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H73" s="14">
+        <f>$B$67-L_x90*$B$69</f>
+        <v/>
+      </c>
+      <c r="I73" s="14">
+        <f>$B$67-L_all90*$B$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>Coupon 19% (cost on receivables = 19% × advance + frictions)</t>
         </is>
       </c>
-      <c r="B73" s="13">
-        <f>$B$66-L_x90*$B$68-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="C73" s="13">
-        <f>$B$66-L_all90*$B$68-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="D73" s="13">
-        <f>$B$66-L_life90x*$B$68-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="E73" s="13">
-        <f>$B$66-L_life90*$B$68-0.19*advance-$B$10</f>
-        <v/>
-      </c>
-      <c r="H73" s="13">
-        <f>$B$66-L_x90*$B$68</f>
-        <v/>
-      </c>
-      <c r="I73" s="13">
-        <f>$B$66-L_all90*$B$68</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74"/>
-    <row r="75">
-      <c r="A75" s="14" t="inlineStr">
+      <c r="B74" s="14">
+        <f>$B$67-L_x90*$B$69-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C74" s="14">
+        <f>$B$67-L_all90*$B$69-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D74" s="14">
+        <f>$B$67-L_life90x*$B$69-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E74" s="14">
+        <f>$B$67-L_life90*$B$69-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="H74" s="14">
+        <f>$B$67-L_x90*$B$69</f>
+        <v/>
+      </c>
+      <c r="I74" s="14">
+        <f>$B$67-L_all90*$B$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75"/>
+    <row r="76">
+      <c r="A76" s="15" t="inlineStr">
         <is>
           <t>Advance rate sensitivity at 19% coupon, base loss — advance →</t>
         </is>
       </c>
-      <c r="B75" s="16" t="n">
+      <c r="B76" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="C75" s="16" t="n">
+      <c r="C76" s="17" t="n">
         <v>0.75</v>
       </c>
-      <c r="D75" s="16" t="n">
+      <c r="D76" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="E75" s="16" t="n">
+      <c r="E76" s="17" t="n">
         <v>0.85</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Excess spread, pts of receivables</t>
-        </is>
-      </c>
-      <c r="B76" s="13">
-        <f>$B$66-L_x90*$B$68-0.19*B75-$B$10</f>
-        <v/>
-      </c>
-      <c r="C76" s="13">
-        <f>$B$66-L_x90*$B$68-0.19*C75-$B$10</f>
-        <v/>
-      </c>
-      <c r="D76" s="13">
-        <f>$B$66-L_x90*$B$68-0.19*D75-$B$10</f>
-        <v/>
-      </c>
-      <c r="E76" s="13">
-        <f>$B$66-L_x90*$B$68-0.19*E75-$B$10</f>
-        <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
-        </is>
-      </c>
-      <c r="B77" s="20">
-        <f>($B$66-L_x90*$B$68)/(0.19*B75+$B$10)</f>
-        <v/>
-      </c>
-      <c r="C77" s="20">
-        <f>($B$66-L_x90*$B$68)/(0.19*C75+$B$10)</f>
-        <v/>
-      </c>
-      <c r="D77" s="20">
-        <f>($B$66-L_x90*$B$68)/(0.19*D75+$B$10)</f>
-        <v/>
-      </c>
-      <c r="E77" s="20">
-        <f>($B$66-L_x90*$B$68)/(0.19*E75+$B$10)</f>
+          <t xml:space="preserve">  Excess spread, pts of receivables</t>
+        </is>
+      </c>
+      <c r="B77" s="14">
+        <f>$B$67-L_x90*$B$69-0.19*B76-s_fric</f>
+        <v/>
+      </c>
+      <c r="C77" s="14">
+        <f>$B$67-L_x90*$B$69-0.19*C76-s_fric</f>
+        <v/>
+      </c>
+      <c r="D77" s="14">
+        <f>$B$67-L_x90*$B$69-0.19*D76-s_fric</f>
+        <v/>
+      </c>
+      <c r="E77" s="14">
+        <f>$B$67-L_x90*$B$69-0.19*E76-s_fric</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Coverage (net yield ÷ cost)</t>
+        </is>
+      </c>
+      <c r="B78" s="21">
+        <f>($B$67-L_x90*$B$69)/(0.19*B76+s_fric)</f>
+        <v/>
+      </c>
+      <c r="C78" s="21">
+        <f>($B$67-L_x90*$B$69)/(0.19*C76+s_fric)</f>
+        <v/>
+      </c>
+      <c r="D78" s="21">
+        <f>($B$67-L_x90*$B$69)/(0.19*D76+s_fric)</f>
+        <v/>
+      </c>
+      <c r="E78" s="21">
+        <f>($B$67-L_x90*$B$69)/(0.19*E76+s_fric)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Breakeven loss rate on originations</t>
         </is>
       </c>
-      <c r="B78" s="18">
-        <f>($B$66-0.19*B75-$B$10)/$B$68</f>
-        <v/>
-      </c>
-      <c r="C78" s="18">
-        <f>($B$66-0.19*C75-$B$10)/$B$68</f>
-        <v/>
-      </c>
-      <c r="D78" s="18">
-        <f>($B$66-0.19*D75-$B$10)/$B$68</f>
-        <v/>
-      </c>
-      <c r="E78" s="18">
-        <f>($B$66-0.19*E75-$B$10)/$B$68</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79"/>
-    <row r="80" ht="64" customHeight="1">
-      <c r="A80" s="21" t="inlineStr">
-        <is>
-          <t>Calibration: the Q3-share block rebuilds revolving interest as rate × scaled revolving balance, so its gross yield (32.1%) sits 0.25 pts under the Q3 sheet (32.4%) and its base-case excess spread reads 5.4 vs 5.6 pts; the gap is the same in every block and does not affect the comparisons. Read across: base case = Q3 share (41.8%), ex-FPD ≥90 loss, 19% coupon, 80% advance → the first cell of the first grid. The second loss column is the tape-level number Accial will compute before any FPD carve-out — at 19% it is close to zero excess spread, which is why FPD ineligibility has to be structural. Moving to 50–60% revolving raises interest yield faster than it dilutes interchange and lowers turnover (so loss on receivables falls): read down the first column of each block. Each 2 pts of coupon ≈ 1.6 pts of excess spread at 80% advance; each 5 pts of advance rate ≈ 1 pt.</t>
+      <c r="B79" s="19">
+        <f>($B$67-0.19*B76-s_fric)/$B$69</f>
+        <v/>
+      </c>
+      <c r="C79" s="19">
+        <f>($B$67-0.19*C76-s_fric)/$B$69</f>
+        <v/>
+      </c>
+      <c r="D79" s="19">
+        <f>($B$67-0.19*D76-s_fric)/$B$69</f>
+        <v/>
+      </c>
+      <c r="E79" s="19">
+        <f>($B$67-0.19*E76-s_fric)/$B$69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80"/>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>Sensitivity — interest-bearing ÷ bucket ratio (growth/timing) at Q3 share, 19% coupon, 80% advance, base loss</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="n"/>
+      <c r="C81" s="5" t="n"/>
+      <c r="D81" s="5" t="n"/>
+      <c r="E81" s="5" t="n"/>
+      <c r="F81" s="5" t="n"/>
+      <c r="G81" s="5" t="n"/>
+      <c r="H81" s="5" t="n"/>
+      <c r="I81" s="5" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="15" t="inlineStr">
+        <is>
+          <t>Ratio →</t>
+        </is>
+      </c>
+      <c r="B82" s="28" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C82" s="28" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D82" s="28" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E82" s="28" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Gross yield — all revenue</t>
+        </is>
+      </c>
+      <c r="B83" s="14">
+        <f>(s_rate*B82*12*$B$14+s_other)/$B$15</f>
+        <v/>
+      </c>
+      <c r="C83" s="14">
+        <f>(s_rate*C82*12*$B$14+s_other)/$B$15</f>
+        <v/>
+      </c>
+      <c r="D83" s="14">
+        <f>(s_rate*D82*12*$B$14+s_other)/$B$15</f>
+        <v/>
+      </c>
+      <c r="E83" s="14">
+        <f>(s_rate*E82*12*$B$14+s_other)/$B$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Excess spread, pts of receivables</t>
+        </is>
+      </c>
+      <c r="B84" s="14">
+        <f>B83-L_x90*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="C84" s="14">
+        <f>C83-L_x90*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="D84" s="14">
+        <f>D83-L_x90*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E84" s="14">
+        <f>E83-L_x90*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="24" t="inlineStr">
+        <is>
+          <t>0.80 is Q3 as observed (book growing ~15%/month). As growth slows the end-of-cycle balance converges on the average revolved balance and the ratio rises; each +0.05 is worth ~0.8 pt of yield at today's revolving share. Pricing is 3.05%/month throughout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86"/>
+    <row r="87" ht="64" customHeight="1">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>Calibration: the Q3-share block rebuilds revolving interest as rate × ratio × scaled revolving balance, so its gross yield (32.1%) sits 0.25 pts under the Q3 sheet (32.4%) and its base-case excess spread reads 5.4 vs 5.6 pts; the gap is the same in every block and does not affect the comparisons. Read across: base case = Q3 share (41.8%), ex-FPD ≥90 loss, 19% coupon, 80% advance → the first cell of the first grid. The second loss column is the tape-level number Accial will compute before any FPD carve-out — at 19% it is close to zero excess spread, which is why FPD ineligibility has to be structural. Moving to 50–60% revolving raises interest yield faster than it dilutes interchange and lowers turnover (so loss on receivables falls): read down the first column of each block. Each 2 pts of coupon ≈ 1.6 pts of excess spread at 80% advance; each 5 pts of advance rate ≈ 1 pt.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A80:I80"/>
+    <mergeCell ref="A87:I87"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3301,7 +3523,7 @@
     </row>
     <row r="2"/>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>KPI Dashboard_v2026 (12).xlsx, Monthly tab</t>
         </is>
@@ -3313,7 +3535,7 @@
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>revolver_transactor_balances_2026-01_to_2026-09_10262026.csv</t>
         </is>
@@ -3325,7 +3547,7 @@
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>vintage_loss_seasoned_16_30_60_90_by_origination_month_10272026.csv (+ .sql)</t>
         </is>
@@ -3337,7 +3559,7 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>vintage_loss_by_origination_month_10262026.csv</t>
         </is>
@@ -3349,7 +3571,7 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>pay_a_friend_transfers_by_month_2026-01_to_2026-09_10272026.csv</t>
         </is>
@@ -3361,7 +3583,7 @@
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Fund-facing counterpart</t>
         </is>
@@ -3373,7 +3595,7 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Annualization</t>
         </is>
@@ -3385,7 +3607,7 @@
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Interchange and loss as turnover functions</t>
         </is>
@@ -3397,7 +3619,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Excluded / placeholders</t>
         </is>
@@ -3409,7 +3631,7 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Prepared</t>
         </is>

</xml_diff>

<commit_message>
Loss emergence by MOB (vintages fully seasoned by ~month 4); recent run-rate loss input L_may26x added to the internal workbook; curves filed
</commit_message>
<xml_diff>
--- a/Analyses (internal)/Facility Yield Analysis_20261027.xlsx
+++ b/Analyses (internal)/Facility Yield Analysis_20261027.xlsx
@@ -40,11 +40,12 @@
     <definedName name="L_life90x">Inputs!$B$33</definedName>
     <definedName name="L_life90">Inputs!$B$34</definedName>
     <definedName name="L_x16">Inputs!$B$35</definedName>
-    <definedName name="coupon">Inputs!$B$37</definedName>
-    <definedName name="advance">Inputs!$B$38</definedName>
-    <definedName name="wht">Inputs!$B$39</definedName>
-    <definedName name="hedge">Inputs!$B$40</definedName>
-    <definedName name="fx">Inputs!$B$41</definedName>
+    <definedName name="L_may26x">Inputs!$B$36</definedName>
+    <definedName name="coupon">Inputs!$B$38</definedName>
+    <definedName name="advance">Inputs!$B$39</definedName>
+    <definedName name="wht">Inputs!$B$40</definedName>
+    <definedName name="hedge">Inputs!$B$41</definedName>
+    <definedName name="fx">Inputs!$B$42</definedName>
     <definedName name="s_rate">Scenarios!$B$5</definedName>
     <definedName name="s_ratio">Scenarios!$B$6</definedName>
     <definedName name="s_share">Scenarios!$B$7</definedName>
@@ -535,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -1312,49 +1313,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>May 2026 vintage, ≥90 DPD, ex-FPD — most recent fully-emerged vintage (RECENT RUN-RATE)</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="n">
+        <v>0.00906</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>source-reports/vintage_loss90_emergence_by_mob_10272026.csv, 2026-05 loss90_xfpd_today_pct</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Loss emergence is complete by ~month 4 on book (FIFO: late defaulters have repaid old tranches), so May 2026 (MOB 5) is effectively final. Fully-emerged ex-FPD by vintage: Jan 2.26% / Feb 1.13% / Mar 1.58% / Apr 1.39% / May 0.91%; Jun 0.34% at MOB 3–4 (≈0.5% when complete). Forward view if FPD → 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>FACILITY ASSUMPTIONS</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="n"/>
-      <c r="E36" s="5" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Coupon (all-in interest on drawn amount)</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>ratio</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Assumption — Steve ('high teens')</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>Scenario grid runs 15/17/19%</t>
-        </is>
-      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Advance rate (drawn ÷ eligible receivables)</t>
+          <t>Coupon (all-in interest on drawn amount)</t>
         </is>
       </c>
       <c r="B38" s="11" t="n">
-        <v>0.8</v>
+        <v>0.19</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1363,23 +1364,23 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Assumption — market 70–85% (structure note §3.3)</t>
+          <t>Assumption — Steve ('high teens')</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Cost of funds on receivables = coupon × advance; scenario runs 70/75/80%</t>
+          <t>Scenario grid runs 15/17/19%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Withholding tax on coupon, if grossed up (placeholder)</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="n">
-        <v>0</v>
+          <t>Advance rate (drawn ÷ eligible receivables)</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="n">
+        <v>0.8</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1388,19 +1389,19 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>NOT SIZED — PH 20% FWT / 15% US treaty (verification-notes/PH tax)</t>
+          <t>Assumption — market 70–85% (structure note §3.3)</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Set to 0 until the structure fixes who bears it; cost if grossed up = coupon × advance × wht ÷ (1 − wht)</t>
+          <t>Cost of funds on receivables = coupon × advance; scenario runs 70/75/80%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FX hedge cost, % of drawn per year (placeholder)</t>
+          <t>Withholding tax on coupon, if grossed up (placeholder)</t>
         </is>
       </c>
       <c r="B40" s="9" t="n">
@@ -1413,35 +1414,60 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>NOT SIZED</t>
+          <t>NOT SIZED — PH 20% FWT / 15% US treaty (verification-notes/PH tax)</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>USD facility vs PHP receivables; PHP/USD forward points — size before pricing</t>
+          <t>Set to 0 until the structure fixes who bears it; cost if grossed up = coupon × advance × wht ÷ (1 − wht)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>FX hedge cost, % of drawn per year (placeholder)</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>NOT SIZED</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>USD facility vs PHP receivables; PHP/USD forward points — size before pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>FX PHP per USD</t>
         </is>
       </c>
-      <c r="B41" s="12" t="n">
+      <c r="B42" s="12" t="n">
         <v>55.8</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>ratio</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D42" s="7" t="inlineStr">
         <is>
           <t>KPI Dashboard Monthly C2</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="E42" s="7" t="inlineStr">
         <is>
           <t>Display only</t>
         </is>
@@ -1781,7 +1807,22 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Loss on receivables at the recent run-rate (May 2026 vintage ex-FPD 0.91% × turnover)</t>
+        </is>
+      </c>
+      <c r="C27" s="14">
+        <f>L_may26x*C21</f>
+        <v/>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Forward view if FPD → 0 and the post-model-change vintages hold; see Inputs L_may26x</t>
+        </is>
+      </c>
+    </row>
     <row r="28"/>
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -2052,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
@@ -2064,6 +2105,8 @@
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2095,6 +2138,8 @@
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2221,6 +2266,8 @@
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n"/>
       <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2296,27 +2343,37 @@
       </c>
       <c r="D20" s="27" t="inlineStr">
         <is>
+          <t>Recent run-rate: May 2026 vintage ex-FPD</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E20" s="27" t="inlineStr">
+      <c r="F20" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
       </c>
-      <c r="G20" s="15" t="inlineStr">
+      <c r="H20" s="15" t="inlineStr">
         <is>
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H20" s="27" t="inlineStr">
+      <c r="I20" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I20" s="27" t="inlineStr">
+      <c r="J20" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
+        </is>
+      </c>
+      <c r="K20" s="27" t="inlineStr">
+        <is>
+          <t>Recent run-rate: May 2026 vintage ex-FPD</t>
         </is>
       </c>
     </row>
@@ -2335,19 +2392,27 @@
         <v/>
       </c>
       <c r="D21" s="14">
+        <f>$B$16-L_may26x*$B$18-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E21" s="14">
         <f>$B$16-L_life90x*$B$18-0.15*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E21" s="14">
+      <c r="F21" s="14">
         <f>$B$16-L_life90*$B$18-0.15*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H21" s="14">
+      <c r="I21" s="14">
         <f>$B$16-L_x90*$B$18</f>
         <v/>
       </c>
-      <c r="I21" s="14">
+      <c r="J21" s="14">
         <f>$B$16-L_all90*$B$18</f>
+        <v/>
+      </c>
+      <c r="K21" s="14">
+        <f>$B$16-L_may26x*$B$18</f>
         <v/>
       </c>
     </row>
@@ -2366,19 +2431,27 @@
         <v/>
       </c>
       <c r="D22" s="14">
+        <f>$B$16-L_may26x*$B$18-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E22" s="14">
         <f>$B$16-L_life90x*$B$18-0.17*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E22" s="14">
+      <c r="F22" s="14">
         <f>$B$16-L_life90*$B$18-0.17*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H22" s="14">
+      <c r="I22" s="14">
         <f>$B$16-L_x90*$B$18</f>
         <v/>
       </c>
-      <c r="I22" s="14">
+      <c r="J22" s="14">
         <f>$B$16-L_all90*$B$18</f>
+        <v/>
+      </c>
+      <c r="K22" s="14">
+        <f>$B$16-L_may26x*$B$18</f>
         <v/>
       </c>
     </row>
@@ -2397,19 +2470,27 @@
         <v/>
       </c>
       <c r="D23" s="14">
+        <f>$B$16-L_may26x*$B$18-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E23" s="14">
         <f>$B$16-L_life90x*$B$18-0.19*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E23" s="14">
+      <c r="F23" s="14">
         <f>$B$16-L_life90*$B$18-0.19*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H23" s="14">
+      <c r="I23" s="14">
         <f>$B$16-L_x90*$B$18</f>
         <v/>
       </c>
-      <c r="I23" s="14">
+      <c r="J23" s="14">
         <f>$B$16-L_all90*$B$18</f>
+        <v/>
+      </c>
+      <c r="K23" s="14">
+        <f>$B$16-L_may26x*$B$18</f>
         <v/>
       </c>
     </row>
@@ -2519,6 +2600,8 @@
       <c r="G30" s="5" t="n"/>
       <c r="H30" s="5" t="n"/>
       <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2594,27 +2677,37 @@
       </c>
       <c r="D37" s="27" t="inlineStr">
         <is>
+          <t>Recent run-rate: May 2026 vintage ex-FPD</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
+        <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E37" s="27" t="inlineStr">
+      <c r="F37" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
       </c>
-      <c r="G37" s="15" t="inlineStr">
+      <c r="H37" s="15" t="inlineStr">
         <is>
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H37" s="27" t="inlineStr">
+      <c r="I37" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I37" s="27" t="inlineStr">
+      <c r="J37" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
+        </is>
+      </c>
+      <c r="K37" s="27" t="inlineStr">
+        <is>
+          <t>Recent run-rate: May 2026 vintage ex-FPD</t>
         </is>
       </c>
     </row>
@@ -2633,19 +2726,27 @@
         <v/>
       </c>
       <c r="D38" s="14">
+        <f>$B$33-L_may26x*$B$35-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E38" s="14">
         <f>$B$33-L_life90x*$B$35-0.15*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E38" s="14">
+      <c r="F38" s="14">
         <f>$B$33-L_life90*$B$35-0.15*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H38" s="14">
+      <c r="I38" s="14">
         <f>$B$33-L_x90*$B$35</f>
         <v/>
       </c>
-      <c r="I38" s="14">
+      <c r="J38" s="14">
         <f>$B$33-L_all90*$B$35</f>
+        <v/>
+      </c>
+      <c r="K38" s="14">
+        <f>$B$33-L_may26x*$B$35</f>
         <v/>
       </c>
     </row>
@@ -2664,19 +2765,27 @@
         <v/>
       </c>
       <c r="D39" s="14">
+        <f>$B$33-L_may26x*$B$35-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E39" s="14">
         <f>$B$33-L_life90x*$B$35-0.17*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E39" s="14">
+      <c r="F39" s="14">
         <f>$B$33-L_life90*$B$35-0.17*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H39" s="14">
+      <c r="I39" s="14">
         <f>$B$33-L_x90*$B$35</f>
         <v/>
       </c>
-      <c r="I39" s="14">
+      <c r="J39" s="14">
         <f>$B$33-L_all90*$B$35</f>
+        <v/>
+      </c>
+      <c r="K39" s="14">
+        <f>$B$33-L_may26x*$B$35</f>
         <v/>
       </c>
     </row>
@@ -2695,19 +2804,27 @@
         <v/>
       </c>
       <c r="D40" s="14">
+        <f>$B$33-L_may26x*$B$35-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E40" s="14">
         <f>$B$33-L_life90x*$B$35-0.19*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E40" s="14">
+      <c r="F40" s="14">
         <f>$B$33-L_life90*$B$35-0.19*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H40" s="14">
+      <c r="I40" s="14">
         <f>$B$33-L_x90*$B$35</f>
         <v/>
       </c>
-      <c r="I40" s="14">
+      <c r="J40" s="14">
         <f>$B$33-L_all90*$B$35</f>
+        <v/>
+      </c>
+      <c r="K40" s="14">
+        <f>$B$33-L_may26x*$B$35</f>
         <v/>
       </c>
     </row>
@@ -2817,6 +2934,8 @@
       <c r="G47" s="5" t="n"/>
       <c r="H47" s="5" t="n"/>
       <c r="I47" s="5" t="n"/>
+      <c r="J47" s="5" t="n"/>
+      <c r="K47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2892,27 +3011,37 @@
       </c>
       <c r="D54" s="27" t="inlineStr">
         <is>
+          <t>Recent run-rate: May 2026 vintage ex-FPD</t>
+        </is>
+      </c>
+      <c r="E54" s="27" t="inlineStr">
+        <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E54" s="27" t="inlineStr">
+      <c r="F54" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
       </c>
-      <c r="G54" s="15" t="inlineStr">
+      <c r="H54" s="15" t="inlineStr">
         <is>
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H54" s="27" t="inlineStr">
+      <c r="I54" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I54" s="27" t="inlineStr">
+      <c r="J54" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
+        </is>
+      </c>
+      <c r="K54" s="27" t="inlineStr">
+        <is>
+          <t>Recent run-rate: May 2026 vintage ex-FPD</t>
         </is>
       </c>
     </row>
@@ -2931,19 +3060,27 @@
         <v/>
       </c>
       <c r="D55" s="14">
+        <f>$B$50-L_may26x*$B$52-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E55" s="14">
         <f>$B$50-L_life90x*$B$52-0.15*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E55" s="14">
+      <c r="F55" s="14">
         <f>$B$50-L_life90*$B$52-0.15*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H55" s="14">
+      <c r="I55" s="14">
         <f>$B$50-L_x90*$B$52</f>
         <v/>
       </c>
-      <c r="I55" s="14">
+      <c r="J55" s="14">
         <f>$B$50-L_all90*$B$52</f>
+        <v/>
+      </c>
+      <c r="K55" s="14">
+        <f>$B$50-L_may26x*$B$52</f>
         <v/>
       </c>
     </row>
@@ -2962,19 +3099,27 @@
         <v/>
       </c>
       <c r="D56" s="14">
+        <f>$B$50-L_may26x*$B$52-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E56" s="14">
         <f>$B$50-L_life90x*$B$52-0.17*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E56" s="14">
+      <c r="F56" s="14">
         <f>$B$50-L_life90*$B$52-0.17*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H56" s="14">
+      <c r="I56" s="14">
         <f>$B$50-L_x90*$B$52</f>
         <v/>
       </c>
-      <c r="I56" s="14">
+      <c r="J56" s="14">
         <f>$B$50-L_all90*$B$52</f>
+        <v/>
+      </c>
+      <c r="K56" s="14">
+        <f>$B$50-L_may26x*$B$52</f>
         <v/>
       </c>
     </row>
@@ -2993,19 +3138,27 @@
         <v/>
       </c>
       <c r="D57" s="14">
+        <f>$B$50-L_may26x*$B$52-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E57" s="14">
         <f>$B$50-L_life90x*$B$52-0.19*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E57" s="14">
+      <c r="F57" s="14">
         <f>$B$50-L_life90*$B$52-0.19*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H57" s="14">
+      <c r="I57" s="14">
         <f>$B$50-L_x90*$B$52</f>
         <v/>
       </c>
-      <c r="I57" s="14">
+      <c r="J57" s="14">
         <f>$B$50-L_all90*$B$52</f>
+        <v/>
+      </c>
+      <c r="K57" s="14">
+        <f>$B$50-L_may26x*$B$52</f>
         <v/>
       </c>
     </row>
@@ -3115,6 +3268,8 @@
       <c r="G64" s="5" t="n"/>
       <c r="H64" s="5" t="n"/>
       <c r="I64" s="5" t="n"/>
+      <c r="J64" s="5" t="n"/>
+      <c r="K64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3190,27 +3345,37 @@
       </c>
       <c r="D71" s="27" t="inlineStr">
         <is>
+          <t>Recent run-rate: May 2026 vintage ex-FPD</t>
+        </is>
+      </c>
+      <c r="E71" s="27" t="inlineStr">
+        <is>
           <t>Lifetime ≥90 ex-FPD</t>
         </is>
       </c>
-      <c r="E71" s="27" t="inlineStr">
+      <c r="F71" s="27" t="inlineStr">
         <is>
           <t>Lifetime ≥90 all accounts</t>
         </is>
       </c>
-      <c r="G71" s="15" t="inlineStr">
+      <c r="H71" s="15" t="inlineStr">
         <is>
           <t>Net yield before funding →</t>
         </is>
       </c>
-      <c r="H71" s="27" t="inlineStr">
+      <c r="I71" s="27" t="inlineStr">
         <is>
           <t>ex-FPD ≥90 since Jan 2026 (BASE)</t>
         </is>
       </c>
-      <c r="I71" s="27" t="inlineStr">
+      <c r="J71" s="27" t="inlineStr">
         <is>
           <t>All accounts ≥90 since Jan 2026</t>
+        </is>
+      </c>
+      <c r="K71" s="27" t="inlineStr">
+        <is>
+          <t>Recent run-rate: May 2026 vintage ex-FPD</t>
         </is>
       </c>
     </row>
@@ -3229,19 +3394,27 @@
         <v/>
       </c>
       <c r="D72" s="14">
+        <f>$B$67-L_may26x*$B$69-0.15*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E72" s="14">
         <f>$B$67-L_life90x*$B$69-0.15*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E72" s="14">
+      <c r="F72" s="14">
         <f>$B$67-L_life90*$B$69-0.15*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H72" s="14">
+      <c r="I72" s="14">
         <f>$B$67-L_x90*$B$69</f>
         <v/>
       </c>
-      <c r="I72" s="14">
+      <c r="J72" s="14">
         <f>$B$67-L_all90*$B$69</f>
+        <v/>
+      </c>
+      <c r="K72" s="14">
+        <f>$B$67-L_may26x*$B$69</f>
         <v/>
       </c>
     </row>
@@ -3260,19 +3433,27 @@
         <v/>
       </c>
       <c r="D73" s="14">
+        <f>$B$67-L_may26x*$B$69-0.17*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E73" s="14">
         <f>$B$67-L_life90x*$B$69-0.17*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E73" s="14">
+      <c r="F73" s="14">
         <f>$B$67-L_life90*$B$69-0.17*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H73" s="14">
+      <c r="I73" s="14">
         <f>$B$67-L_x90*$B$69</f>
         <v/>
       </c>
-      <c r="I73" s="14">
+      <c r="J73" s="14">
         <f>$B$67-L_all90*$B$69</f>
+        <v/>
+      </c>
+      <c r="K73" s="14">
+        <f>$B$67-L_may26x*$B$69</f>
         <v/>
       </c>
     </row>
@@ -3291,19 +3472,27 @@
         <v/>
       </c>
       <c r="D74" s="14">
+        <f>$B$67-L_may26x*$B$69-0.19*advance-s_fric</f>
+        <v/>
+      </c>
+      <c r="E74" s="14">
         <f>$B$67-L_life90x*$B$69-0.19*advance-s_fric</f>
         <v/>
       </c>
-      <c r="E74" s="14">
+      <c r="F74" s="14">
         <f>$B$67-L_life90*$B$69-0.19*advance-s_fric</f>
         <v/>
       </c>
-      <c r="H74" s="14">
+      <c r="I74" s="14">
         <f>$B$67-L_x90*$B$69</f>
         <v/>
       </c>
-      <c r="I74" s="14">
+      <c r="J74" s="14">
         <f>$B$67-L_all90*$B$69</f>
+        <v/>
+      </c>
+      <c r="K74" s="14">
+        <f>$B$67-L_may26x*$B$69</f>
         <v/>
       </c>
     </row>
@@ -3411,6 +3600,8 @@
       <c r="G81" s="5" t="n"/>
       <c r="H81" s="5" t="n"/>
       <c r="I81" s="5" t="n"/>
+      <c r="J81" s="5" t="n"/>
+      <c r="K81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="15" t="inlineStr">
@@ -3494,8 +3685,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A87:I87"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A87:K87"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>